<commit_message>
chore: remove legacy dashboard and planning tool files and update primary planning tool version
</commit_message>
<xml_diff>
--- a/TOPSIM_Planungstool_V8.xlsx
+++ b/TOPSIM_Planungstool_V8.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Bastian\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\FinancePlanningTool_BusinessSimulation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDD64D7D-46B5-4EC3-A454-6B598D66D1CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6DCD058-14E1-4FED-A04B-531A236202CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TOPSIM Planung" sheetId="1" r:id="rId1"/>
@@ -210,7 +210,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -231,8 +231,15 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C5700"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -254,6 +261,11 @@
         <fgColor rgb="FFDCE6F1"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -264,10 +276,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -276,8 +289,10 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Neutral" xfId="1" builtinId="28"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -579,13 +594,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B61"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="65" customWidth="1"/>
     <col min="2" max="2" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -593,38 +608,38 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="2"/>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="3">
-        <v>45000</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+        <v>43000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="3">
-        <v>3200</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+        <v>3150</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>5</v>
       </c>
       <c r="B5" s="4">
         <f>B3*B4/1000000</f>
-        <v>144</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+        <v>135.44999999999999</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -632,7 +647,7 @@
         <v>-95</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -640,7 +655,7 @@
         <v>-3.5</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -648,7 +663,7 @@
         <v>-26.5</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -656,7 +671,7 @@
         <v>-20</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>10</v>
       </c>
@@ -664,15 +679,15 @@
         <v>-6.75</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A11" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="3">
+      <c r="B11" s="6">
         <v>-0.25</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -680,32 +695,32 @@
         <v>-2.5</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>13</v>
       </c>
       <c r="B13" s="5">
         <f>SUM(B5:B12)</f>
-        <v>-10.5</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
+        <v>-19.050000000000011</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A14" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B14" s="3">
+      <c r="B14" s="6">
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A15" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="3">
+      <c r="B15" s="6">
         <v>8</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>16</v>
       </c>
@@ -713,7 +728,7 @@
         <v>25.5</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>17</v>
       </c>
@@ -721,7 +736,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>18</v>
       </c>
@@ -730,16 +745,16 @@
         <v>-2.585</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>19</v>
       </c>
       <c r="B19" s="5">
         <f>B13+B18</f>
-        <v>-13.085000000000001</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+        <v>-21.635000000000012</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>20</v>
       </c>
@@ -747,7 +762,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>21</v>
       </c>
@@ -756,15 +771,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A22" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B22" s="3">
+      <c r="B22" s="6">
         <v>45</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
         <v>23</v>
       </c>
@@ -773,22 +788,22 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>24</v>
       </c>
       <c r="B24" s="5">
         <f>B19+B23</f>
-        <v>-13.085000000000001</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+        <v>-21.635000000000012</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>25</v>
       </c>
       <c r="B26" s="2"/>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>26</v>
       </c>
@@ -796,7 +811,7 @@
         <v>43.02</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>27</v>
       </c>
@@ -804,39 +819,39 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
         <v>28</v>
       </c>
       <c r="B29" s="5">
         <f>B27+B28+B24</f>
-        <v>28.935000000000002</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+        <v>20.384999999999991</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>29</v>
       </c>
       <c r="B30" s="5">
         <f>(B24/B29)*100</f>
-        <v>-45.222049421116296</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+        <v>-106.131959774344</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
         <v>31</v>
       </c>
       <c r="B33" s="5">
         <f>B24</f>
-        <v>-13.085000000000001</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+        <v>-21.635000000000012</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>32</v>
       </c>
@@ -845,7 +860,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>33</v>
       </c>
@@ -853,16 +868,16 @@
         <v>2</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>34</v>
       </c>
       <c r="B36" s="4">
         <f>B33+B34+B35</f>
-        <v>-1.5850000000000009</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+        <v>-10.135000000000012</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>35</v>
       </c>
@@ -870,7 +885,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>36</v>
       </c>
@@ -878,36 +893,36 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
         <v>37</v>
       </c>
       <c r="B39" s="5">
         <f>B36+B37+B38</f>
-        <v>-3.5850000000000009</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+        <v>-12.135000000000012</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
         <v>38</v>
       </c>
       <c r="B41" s="2"/>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>40</v>
       </c>
       <c r="B43" s="4">
         <f>B5*0.8</f>
-        <v>115.2</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+        <v>108.36</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>41</v>
       </c>
@@ -915,7 +930,7 @@
         <v>25.8</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>42</v>
       </c>
@@ -923,21 +938,21 @@
         <v>30</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>43</v>
       </c>
       <c r="B46" s="4">
         <f>SUM(B43:B45)</f>
-        <v>171</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+        <v>164.16</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A48" s="2" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>45</v>
       </c>
@@ -946,7 +961,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>46</v>
       </c>
@@ -955,7 +970,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>47</v>
       </c>
@@ -964,7 +979,7 @@
         <v>46.5</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>48</v>
       </c>
@@ -973,7 +988,7 @@
         <v>2.585</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>49</v>
       </c>
@@ -982,7 +997,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>50</v>
       </c>
@@ -990,7 +1005,7 @@
         <v>22.5</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>51</v>
       </c>
@@ -998,7 +1013,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>52</v>
       </c>
@@ -1007,7 +1022,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>53</v>
       </c>
@@ -1016,16 +1031,16 @@
         <v>191.08500000000001</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>54</v>
       </c>
       <c r="B59" s="4">
         <f>B46-B57</f>
-        <v>-20.085000000000008</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
+        <v>-26.925000000000011</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>55</v>
       </c>
@@ -1033,13 +1048,13 @@
         <v>11.26</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A61" s="2" t="s">
         <v>56</v>
       </c>
       <c r="B61" s="4">
         <f>B59+B60</f>
-        <v>-8.8250000000000082</v>
+        <v>-15.665000000000012</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update business simulation parameters in TOPSIM_Planungstool_V8.xlsx
</commit_message>
<xml_diff>
--- a/TOPSIM_Planungstool_V8.xlsx
+++ b/TOPSIM_Planungstool_V8.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\FinancePlanningTool_BusinessSimulation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6DCD058-14E1-4FED-A04B-531A236202CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0260A73-BE77-4A78-B400-87855D76B609}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,14 +33,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="59">
   <si>
     <t>Position</t>
   </si>
   <si>
-    <t>Szenario 1 (Planung)</t>
-  </si>
-  <si>
     <t>1. PLAN-GEWINN- UND VERLUSTRECHNUNG</t>
   </si>
   <si>
@@ -204,6 +201,15 @@
   </si>
   <si>
     <t>ZAHLUNGSMITTELENDBESTAND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Szenario 1 </t>
+  </si>
+  <si>
+    <t>25,8-27,09</t>
+  </si>
+  <si>
+    <t>(7,91-7,15)+0</t>
   </si>
 </sst>
 </file>
@@ -219,27 +225,28 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color rgb="FF9C5700"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -248,22 +255,34 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF4F81BD"/>
+        <fgColor rgb="FFFFEB9C"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEBF1DE"/>
+        <fgColor theme="4"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFDCE6F1"/>
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
+        <fgColor theme="6" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
       </patternFill>
     </fill>
   </fills>
@@ -276,22 +295,32 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="5" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="4"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="3"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="6"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="7">
+    <cellStyle name="60 % - Akzent1" xfId="3" builtinId="32"/>
+    <cellStyle name="60 % - Akzent3" xfId="4" builtinId="40"/>
+    <cellStyle name="Akzent1" xfId="2" builtinId="29"/>
+    <cellStyle name="Akzent4" xfId="5" builtinId="41"/>
+    <cellStyle name="Akzent5" xfId="6" builtinId="45"/>
     <cellStyle name="Neutral" xfId="1" builtinId="28"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
@@ -593,195 +622,198 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B61"/>
+  <dimension ref="A1:C61"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="65" customWidth="1"/>
     <col min="2" max="2" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
+      <c r="B2" s="2"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2"/>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+      <c r="B3" s="4">
+        <v>43000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="3">
-        <v>43000</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
+      <c r="B4" s="4">
+        <v>3150</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="3">
-        <v>3150</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="4">
+      <c r="B5" s="5">
         <f>B3*B4/1000000</f>
         <v>135.44999999999999</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4">
+        <v>-98</v>
+      </c>
+      <c r="C6" s="4">
+        <v>-38.96</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="3">
-        <v>-95</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
+      <c r="B7" s="4">
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="3">
-        <v>-3.5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
+      <c r="B8" s="4">
+        <v>-10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="3">
-        <v>-26.5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
+      <c r="B9" s="4">
+        <v>-8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="3">
-        <v>-20</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
+      <c r="B10" s="4">
+        <v>-6.75</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="3">
-        <v>-6.75</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A11" s="6" t="s">
+      <c r="B11" s="1">
+        <v>-0.25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="6">
-        <v>-0.25</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
+      <c r="B12" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" s="5" t="s">
         <v>12</v>
-      </c>
-      <c r="B12" s="3">
-        <v>-2.5</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A13" s="2" t="s">
-        <v>13</v>
       </c>
       <c r="B13" s="5">
         <f>SUM(B5:B12)</f>
-        <v>-19.050000000000011</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A14" s="6" t="s">
+        <v>7.4499999999999886</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B14" s="6">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A15" s="6" t="s">
+      <c r="B15" s="1">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="6">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
+      <c r="B16" s="4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A17" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="3">
-        <v>25.5</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
+      <c r="B17" s="4">
         <v>17</v>
       </c>
-      <c r="B17" s="3">
-        <v>10</v>
-      </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A18" s="2" t="s">
-        <v>18</v>
+      <c r="A18" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B18" s="5">
         <f>-(B16*(B14/100) + B17*(B15/100))</f>
-        <v>-2.585</v>
+        <v>-1.7100000000000002</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A19" s="2" t="s">
-        <v>19</v>
+      <c r="A19" s="5" t="s">
+        <v>18</v>
       </c>
       <c r="B19" s="5">
         <f>B13+B18</f>
-        <v>-21.635000000000012</v>
+        <v>5.7399999999999887</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
+      <c r="A20" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B20" s="4">
+        <v>6.27</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A21" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B20" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
-        <v>21</v>
-      </c>
-      <c r="B21" s="4">
+      <c r="B21" s="5">
         <f>MAX(0, B19-B20)</f>
         <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A22" s="6" t="s">
+      <c r="A22" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22" s="1">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A23" s="5" t="s">
         <v>22</v>
-      </c>
-      <c r="B22" s="6">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A23" s="2" t="s">
-        <v>23</v>
       </c>
       <c r="B23" s="5">
         <f>-B21*(B22/100)</f>
@@ -789,272 +821,283 @@
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A24" s="2" t="s">
-        <v>24</v>
+      <c r="A24" s="5" t="s">
+        <v>23</v>
       </c>
       <c r="B24" s="5">
         <f>B19+B23</f>
-        <v>-21.635000000000012</v>
+        <v>5.7399999999999887</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B26" s="2"/>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A27" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B26" s="2"/>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
+      <c r="B27" s="4">
+        <v>31.27</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A28" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B27" s="3">
-        <v>43.02</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
+      <c r="B28" s="4">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A29" s="5" t="s">
         <v>27</v>
-      </c>
-      <c r="B28" s="3">
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A29" s="2" t="s">
-        <v>28</v>
       </c>
       <c r="B29" s="5">
         <f>B27+B28+B24</f>
-        <v>20.384999999999991</v>
+        <v>36.009999999999991</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A30" s="2" t="s">
-        <v>29</v>
+      <c r="A30" s="5" t="s">
+        <v>28</v>
       </c>
       <c r="B30" s="5">
         <f>(B24/B29)*100</f>
-        <v>-106.131959774344</v>
+        <v>15.940016662038294</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A32" t="s">
+      <c r="A32" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B32" s="2"/>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A33" s="5" t="s">
         <v>30</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A33" s="2" t="s">
-        <v>31</v>
       </c>
       <c r="B33" s="5">
         <f>B24</f>
-        <v>-21.635000000000012</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
+        <v>5.7399999999999887</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A34" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B34" s="5">
+        <f>-(B10+B11+B12)</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A35" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B34" s="4">
-        <f>-(B10+B11+B12)</f>
-        <v>9.5</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A35" t="s">
+      <c r="B35" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A36" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B35" s="3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A36" t="s">
+      <c r="B36" s="5">
+        <f>B33+B34+B35</f>
+        <v>14.739999999999988</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A37" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="B36" s="4">
-        <f>B33+B34+B35</f>
-        <v>-10.135000000000012</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A37" t="s">
+      <c r="B37" s="4">
+        <f>25.8-27.09</f>
+        <v>-1.2899999999999991</v>
+      </c>
+      <c r="C37" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A38" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="B37" s="3">
-        <v>-3</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A38" t="s">
+      <c r="B38" s="4">
+        <f>(7.91-7.15)+0</f>
+        <v>0.75999999999999979</v>
+      </c>
+      <c r="C38" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A39" s="5" t="s">
         <v>36</v>
-      </c>
-      <c r="B38" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A39" s="2" t="s">
-        <v>37</v>
       </c>
       <c r="B39" s="5">
         <f>B36+B37+B38</f>
-        <v>-12.135000000000012</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+        <v>14.209999999999988</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B41" s="2"/>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A42" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="B41" s="2"/>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A42" s="2" t="s">
+      <c r="B42" s="6"/>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A43" s="5" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A43" t="s">
-        <v>40</v>
-      </c>
-      <c r="B43" s="4">
+      <c r="B43" s="5">
         <f>B5*0.8</f>
         <v>108.36</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A44" t="s">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A44" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B44" s="4">
+        <v>25.8</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A45" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="B44" s="3">
-        <v>25.8</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A45" t="s">
+      <c r="B45" s="4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A46" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="B45" s="3">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A46" t="s">
+      <c r="B46" s="5">
+        <f>SUM(B43:B45)</f>
+        <v>156.16</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A48" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="B46" s="4">
-        <f>SUM(B43:B45)</f>
-        <v>164.16</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A48" s="2" t="s">
+      <c r="B48" s="6"/>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A49" s="5" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A49" t="s">
+      <c r="B49" s="5">
+        <f>-B6</f>
+        <v>98</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A50" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="B49" s="4">
-        <f>-B6</f>
-        <v>95</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A50" t="s">
+      <c r="B50" s="5">
+        <f>-B7</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A51" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="B50" s="4">
-        <f>-B7</f>
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A51" t="s">
+      <c r="B51" s="5">
+        <f>-(B8+B9)</f>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A52" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="B51" s="4">
-        <f>-(B8+B9)</f>
-        <v>46.5</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A52" t="s">
+      <c r="B52" s="5">
+        <f>-B18</f>
+        <v>1.7100000000000002</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A53" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="B52" s="4">
-        <f>-B18</f>
-        <v>2.585</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A53" t="s">
-        <v>49</v>
-      </c>
-      <c r="B53" s="4">
+      <c r="B53" s="5">
         <f>-B23</f>
         <v>0</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A54" t="s">
+      <c r="A54" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B54" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A55" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="B54" s="3">
-        <v>22.5</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A55" t="s">
+      <c r="B55" s="4">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A56" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="B55" s="3">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A56" t="s">
-        <v>52</v>
-      </c>
-      <c r="B56" s="4">
+      <c r="B56" s="5">
         <f>-B28</f>
         <v>1</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A57" t="s">
+      <c r="A57" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B57" s="5">
+        <f>SUM(B49:B56)</f>
+        <v>150.70999999999998</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A59" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B57" s="4">
-        <f>SUM(B49:B56)</f>
-        <v>191.08500000000001</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A59" t="s">
+      <c r="B59" s="5">
+        <f>B46-B57</f>
+        <v>5.4500000000000171</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A60" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B59" s="4">
-        <f>B46-B57</f>
-        <v>-26.925000000000011</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A60" t="s">
+      <c r="B60" s="4">
+        <v>11.26</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A61" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="B60" s="3">
-        <v>11.26</v>
-      </c>
-    </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A61" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="B61" s="4">
+      <c r="B61" s="5">
         <f>B59+B60</f>
-        <v>-15.665000000000012</v>
+        <v>16.710000000000015</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated to the second period
</commit_message>
<xml_diff>
--- a/TOPSIM_Planungstool_V8.xlsx
+++ b/TOPSIM_Planungstool_V8.xlsx
@@ -5,15 +5,18 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\FinancePlanningTool_BusinessSimulation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/96db5acea2ea2686/Hochschule/Sechstes Semester/Business Simulation/Finance Tool/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0260A73-BE77-4A78-B400-87855D76B609}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="147" documentId="13_ncr:1_{E0260A73-BE77-4A78-B400-87855D76B609}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2A480106-1B4A-4CBD-AFC2-DB88121606B6}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="17496" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="TOPSIM Planung" sheetId="1" r:id="rId1"/>
+    <sheet name="Formeln" sheetId="3" r:id="rId1"/>
+    <sheet name="Periode 1" sheetId="1" r:id="rId2"/>
+    <sheet name="Periode 2" sheetId="2" r:id="rId3"/>
+    <sheet name="Periode 3" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="69">
   <si>
     <t>Position</t>
   </si>
@@ -210,13 +213,49 @@
   </si>
   <si>
     <t>(7,91-7,15)+0</t>
+  </si>
+  <si>
+    <t>HIER 0 EINTRAGEN</t>
+  </si>
+  <si>
+    <t>Kommentar</t>
+  </si>
+  <si>
+    <t>F&amp;E-Kosten (GuV) = F&amp;E-Mitarbeiter × Gehalt × (1 + PNK%)
+                   + Einstellungs-/Entlassungskosten
+                   + Pensionsrückstellungen (anteilig)
+                   + Gebäude-Abschreibung (5%)
+                   + Ökologie-Budget
+                   + Wertanalyse-Budget</t>
+  </si>
+  <si>
+    <t>Kreditaufnahme Summe</t>
+  </si>
+  <si>
+    <t>Kreditaufnahme NEU Langfristig</t>
+  </si>
+  <si>
+    <t>Forderungen Vorperiode</t>
+  </si>
+  <si>
+    <t>Veränderung Vorräte = Δ Materialien + Δ Fertige Erzeugnisse</t>
+  </si>
+  <si>
+    <t>Material-Lager (neu) = Material-Lager (alt) + Einkauf − Verbrauch
+Verbrauch            ≈ Fertigungsmenge × Materialkosten pro Stück / Wertanalyseindex</t>
+  </si>
+  <si>
+    <t>Lager FE (neu) = Lager FE (alt) + Produktion − Absatz   (in Stück, bewertet zu Herstellkosten)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Material: 40500+2843-47000 = -157; Lager: 43500+5858-47000 = 2358 </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -241,6 +280,19 @@
     <font>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -304,7 +356,7 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="2"/>
@@ -314,6 +366,11 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="4"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="3"/>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="6"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="4" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="60 % - Akzent1" xfId="3" builtinId="32"/>
@@ -335,6 +392,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -621,15 +682,48 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C98663D-40D0-402A-B2D8-812995C4C756}">
+  <dimension ref="A1:A5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="39.109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A1" s="9" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="9" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="9" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A5" s="9" t="s">
+        <v>67</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C61"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="65" customWidth="1"/>
     <col min="2" max="2" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -637,13 +731,13 @@
         <v>56</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="2"/>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
@@ -651,7 +745,7 @@
         <v>43000</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
@@ -659,7 +753,7 @@
         <v>3150</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>4</v>
       </c>
@@ -668,7 +762,7 @@
         <v>135.44999999999999</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>5</v>
       </c>
@@ -679,7 +773,7 @@
         <v>-38.96</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>6</v>
       </c>
@@ -687,7 +781,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>7</v>
       </c>
@@ -695,7 +789,7 @@
         <v>-10</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>8</v>
       </c>
@@ -703,7 +797,7 @@
         <v>-8</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>9</v>
       </c>
@@ -711,7 +805,7 @@
         <v>-6.75</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>10</v>
       </c>
@@ -719,7 +813,7 @@
         <v>-0.25</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>11</v>
       </c>
@@ -727,7 +821,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
         <v>12</v>
       </c>
@@ -736,7 +830,7 @@
         <v>7.4499999999999886</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>13</v>
       </c>
@@ -744,7 +838,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>14</v>
       </c>
@@ -752,7 +846,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>15</v>
       </c>
@@ -760,7 +854,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
         <v>16</v>
       </c>
@@ -768,7 +862,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
         <v>17</v>
       </c>
@@ -777,7 +871,7 @@
         <v>-1.7100000000000002</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
         <v>18</v>
       </c>
@@ -786,24 +880,27 @@
         <v>5.7399999999999887</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B20" s="4">
-        <v>6.27</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B20" s="8">
+        <v>0</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
         <v>20</v>
       </c>
       <c r="B21" s="5">
         <f>MAX(0, B19-B20)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+        <v>5.7399999999999887</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>21</v>
       </c>
@@ -811,31 +908,31 @@
         <v>45</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
         <v>22</v>
       </c>
       <c r="B23" s="5">
         <f>-B21*(B22/100)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+        <v>-2.5829999999999949</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
         <v>23</v>
       </c>
       <c r="B24" s="5">
         <f>B19+B23</f>
-        <v>5.7399999999999887</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+        <v>3.1569999999999938</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>24</v>
       </c>
       <c r="B26" s="2"/>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
         <v>25</v>
       </c>
@@ -843,7 +940,7 @@
         <v>31.27</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
         <v>26</v>
       </c>
@@ -851,40 +948,40 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="s">
         <v>27</v>
       </c>
       <c r="B29" s="5">
         <f>B27+B28+B24</f>
-        <v>36.009999999999991</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+        <v>33.426999999999992</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" s="5" t="s">
         <v>28</v>
       </c>
       <c r="B30" s="5">
         <f>(B24/B29)*100</f>
-        <v>15.940016662038294</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+        <v>9.4444610644089941</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>29</v>
       </c>
       <c r="B32" s="2"/>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" s="5" t="s">
         <v>30</v>
       </c>
       <c r="B33" s="5">
         <f>B24</f>
-        <v>5.7399999999999887</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+        <v>3.1569999999999938</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" s="5" t="s">
         <v>31</v>
       </c>
@@ -893,7 +990,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
         <v>32</v>
       </c>
@@ -901,16 +998,16 @@
         <v>2</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" s="5" t="s">
         <v>33</v>
       </c>
       <c r="B36" s="5">
         <f>B33+B34+B35</f>
-        <v>14.739999999999988</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+        <v>12.156999999999993</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
         <v>34</v>
       </c>
@@ -922,7 +1019,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
         <v>35</v>
       </c>
@@ -934,28 +1031,28 @@
         <v>58</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" s="5" t="s">
         <v>36</v>
       </c>
       <c r="B39" s="5">
         <f>B36+B37+B38</f>
-        <v>14.209999999999988</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+        <v>11.626999999999994</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>37</v>
       </c>
       <c r="B41" s="2"/>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" s="6" t="s">
         <v>38</v>
       </c>
       <c r="B42" s="6"/>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43" s="5" t="s">
         <v>39</v>
       </c>
@@ -964,7 +1061,7 @@
         <v>108.36</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
         <v>40</v>
       </c>
@@ -972,7 +1069,7 @@
         <v>25.8</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45" s="4" t="s">
         <v>41</v>
       </c>
@@ -980,7 +1077,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46" s="5" t="s">
         <v>42</v>
       </c>
@@ -989,13 +1086,13 @@
         <v>156.16</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A48" s="6" t="s">
         <v>43</v>
       </c>
       <c r="B48" s="6"/>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A49" s="5" t="s">
         <v>44</v>
       </c>
@@ -1004,7 +1101,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A50" s="5" t="s">
         <v>45</v>
       </c>
@@ -1013,7 +1110,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A51" s="5" t="s">
         <v>46</v>
       </c>
@@ -1022,7 +1119,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" s="5" t="s">
         <v>47</v>
       </c>
@@ -1031,16 +1128,16 @@
         <v>1.7100000000000002</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A53" s="5" t="s">
         <v>48</v>
       </c>
       <c r="B53" s="5">
         <f>-B23</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+        <v>2.5829999999999949</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A54" s="4" t="s">
         <v>49</v>
       </c>
@@ -1048,7 +1145,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A55" s="4" t="s">
         <v>50</v>
       </c>
@@ -1056,7 +1153,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A56" s="5" t="s">
         <v>51</v>
       </c>
@@ -1065,25 +1162,25 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A57" s="5" t="s">
         <v>52</v>
       </c>
       <c r="B57" s="5">
         <f>SUM(B49:B56)</f>
-        <v>150.70999999999998</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
+        <v>153.29300000000001</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A59" s="5" t="s">
         <v>53</v>
       </c>
       <c r="B59" s="5">
         <f>B46-B57</f>
-        <v>5.4500000000000171</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
+        <v>2.8669999999999902</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A60" s="4" t="s">
         <v>54</v>
       </c>
@@ -1091,16 +1188,1026 @@
         <v>11.26</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A61" s="5" t="s">
         <v>55</v>
       </c>
       <c r="B61" s="5">
         <f>B59+B60</f>
-        <v>16.710000000000015</v>
+        <v>14.12699999999999</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="4294967293" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3670D53-6421-4BCC-8263-1590D4CFD838}">
+  <dimension ref="A1:C63"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="65" customWidth="1"/>
+    <col min="2" max="2" width="25" customWidth="1"/>
+    <col min="3" max="3" width="13.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4">
+        <v>47000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4">
+        <v>3200</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="5">
+        <f>B3*B4/1000000</f>
+        <v>150.4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4">
+        <v>-95</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4">
+        <v>-7.1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="4">
+        <v>-10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="4">
+        <v>-20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="4">
+        <v>-6.75</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="1">
+        <v>-0.25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="5">
+        <f>SUM(B5:B12)</f>
+        <v>11.300000000000004</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" s="1">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" s="4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17" s="4">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18" s="5">
+        <f>-(B16*(B14/100) + B17*(B15/100))</f>
+        <v>-1.31</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" s="5">
+        <f>B13+B18</f>
+        <v>9.9900000000000038</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B20" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" s="5">
+        <f>MAX(0, B19-B20)</f>
+        <v>9.9900000000000038</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A22" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22" s="1">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A23" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B23" s="5">
+        <f>-B21*(B22/100)</f>
+        <v>-4.4955000000000016</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A24" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B24" s="5">
+        <f>B19+B23</f>
+        <v>5.4945000000000022</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A26" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B26" s="2"/>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A27" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B27" s="4">
+        <v>35.03</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A28" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B28" s="4">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A29" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B29" s="5">
+        <f>B27+B28+B24</f>
+        <v>39.524500000000003</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A30" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B30" s="5">
+        <f>(B24/B29)*100</f>
+        <v>13.901504130349535</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A32" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B32" s="2"/>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B33" s="5">
+        <f>B24</f>
+        <v>5.4945000000000022</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B34" s="5">
+        <f>-(B10+B11+B12)</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B35" s="4">
+        <v>2.2000000000000002</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B36" s="5">
+        <f>B33+B34+B35</f>
+        <v>14.694500000000001</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B37" s="4">
+        <v>26.72</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A38" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B38" s="4">
+        <f>B5*0.2-B37</f>
+        <v>3.360000000000003</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B39" s="4">
+        <f>4.8</f>
+        <v>4.8</v>
+      </c>
+      <c r="C39" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A40" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B40" s="5">
+        <f>B36+B38+B39</f>
+        <v>22.854500000000005</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A42" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B42" s="2"/>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A43" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B43" s="6"/>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A44" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B44" s="5">
+        <f>B5*0.8</f>
+        <v>120.32000000000001</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A45" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B45" s="4">
+        <v>25.8</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A46" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B46" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A47" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="B47" s="4">
+        <f>B46+B17</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A48" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B48" s="5">
+        <f>B44+B45+B47</f>
+        <v>158.12</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A50" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B50" s="6"/>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A51" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B51" s="5">
+        <f>-B6</f>
+        <v>95</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A52" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="B52" s="5">
+        <f>-B7</f>
+        <v>7.1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A53" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="B53" s="5">
+        <f>-(B8+B9)</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A54" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B54" s="5">
+        <f>-B18</f>
+        <v>1.31</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A55" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B55" s="5">
+        <f>-B23</f>
+        <v>4.4955000000000016</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A56" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B56" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A57" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B57" s="4">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A58" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B58" s="5">
+        <f>-B28</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A59" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B59" s="5">
+        <f>SUM(B51:B58)</f>
+        <v>155.90549999999999</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A61" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B61" s="5">
+        <f>B48-B59</f>
+        <v>2.2145000000000152</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A62" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B62" s="4">
+        <v>11.26</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A63" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B63" s="5">
+        <f>B61+B62</f>
+        <v>13.474500000000015</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="4294967293" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CDA27C3-61FD-40B5-8531-C2A107CE4E67}">
+  <dimension ref="A1:C63"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="65" customWidth="1"/>
+    <col min="2" max="2" width="25" customWidth="1"/>
+    <col min="3" max="3" width="13.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4">
+        <v>47000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4">
+        <v>3200</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="5">
+        <f>B3*B4/1000000</f>
+        <v>150.4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4">
+        <v>-93</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4">
+        <v>-7.1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="4">
+        <v>-10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="4">
+        <v>-20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="4">
+        <v>-6.75</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="1">
+        <v>-0.25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="5">
+        <f>SUM(B5:B12)</f>
+        <v>13.300000000000004</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="1">
+        <v>6</v>
+      </c>
+      <c r="C14">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" s="1">
+        <v>7</v>
+      </c>
+      <c r="C15">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" s="4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17" s="4">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18" s="5">
+        <f>-(B16*(B14/100) + B17*(B15/100))</f>
+        <v>-1.1400000000000001</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" s="5">
+        <f>B13+B18</f>
+        <v>12.160000000000004</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B20" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" s="5">
+        <f>MAX(0, B19-B20)</f>
+        <v>12.160000000000004</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A22" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22" s="1">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A23" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B23" s="5">
+        <f>-B21*(B22/100)</f>
+        <v>-5.4720000000000022</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A24" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B24" s="5">
+        <f>B19+B23</f>
+        <v>6.6880000000000015</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A26" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B26" s="2"/>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A27" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B27" s="4">
+        <v>35.03</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A28" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B28" s="4">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A29" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B29" s="5">
+        <f>B27+B28+B24</f>
+        <v>40.718000000000004</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A30" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B30" s="5">
+        <f>(B24/B27)*100</f>
+        <v>19.092206679988585</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A32" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B32" s="2"/>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B33" s="5">
+        <f>B24</f>
+        <v>6.6880000000000015</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B34" s="5">
+        <f>-(B10+B11+B12)</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B35" s="4">
+        <v>2.2000000000000002</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B36" s="5">
+        <f>B33+B34+B35</f>
+        <v>15.888000000000002</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B37" s="4">
+        <v>26.72</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A38" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B38" s="4">
+        <f>B5*0.2-B37</f>
+        <v>3.360000000000003</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B39" s="4">
+        <f>4.8</f>
+        <v>4.8</v>
+      </c>
+      <c r="C39" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A40" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B40" s="5">
+        <f>B36+B38+B39</f>
+        <v>24.048000000000005</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A42" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B42" s="2"/>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A43" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B43" s="6"/>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A44" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B44" s="5">
+        <f>B5*0.8</f>
+        <v>120.32000000000001</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A45" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B45" s="4">
+        <v>25.8</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A46" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B46" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A47" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="B47" s="4">
+        <f>B46+B17</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A48" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B48" s="5">
+        <f>B44+B45+B47</f>
+        <v>158.12</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A50" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B50" s="6"/>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A51" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B51" s="5">
+        <f>-B6</f>
+        <v>93</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A52" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="B52" s="5">
+        <f>-B7</f>
+        <v>7.1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A53" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="B53" s="5">
+        <f>-(B8+B9)</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A54" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B54" s="5">
+        <f>-B18</f>
+        <v>1.1400000000000001</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A55" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B55" s="5">
+        <f>-B23</f>
+        <v>5.4720000000000022</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A56" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B56" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A57" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B57" s="4">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A58" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B58" s="5">
+        <f>-B28</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A59" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B59" s="5">
+        <f>SUM(B51:B58)</f>
+        <v>154.71199999999999</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A61" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B61" s="5">
+        <f>B48-B59</f>
+        <v>3.4080000000000155</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A62" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B62" s="4">
+        <v>11.26</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A63" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B63" s="5">
+        <f>B61+B62</f>
+        <v>14.668000000000015</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="4294967293" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated to thrid period
</commit_message>
<xml_diff>
--- a/TOPSIM_Planungstool_V8.xlsx
+++ b/TOPSIM_Planungstool_V8.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/96db5acea2ea2686/Hochschule/Sechstes Semester/Business Simulation/Finance Tool/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="147" documentId="13_ncr:1_{E0260A73-BE77-4A78-B400-87855D76B609}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2A480106-1B4A-4CBD-AFC2-DB88121606B6}"/>
+  <xr:revisionPtr revIDLastSave="170" documentId="13_ncr:1_{E0260A73-BE77-4A78-B400-87855D76B609}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DFDC3F65-21B4-4C2E-A002-569A580669EB}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="17496" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="70">
   <si>
     <t>Position</t>
   </si>
@@ -249,6 +249,9 @@
   </si>
   <si>
     <t xml:space="preserve">Material: 40500+2843-47000 = -157; Lager: 43500+5858-47000 = 2358 </t>
+  </si>
+  <si>
+    <t>Im Moment noch 6 aber bei Neuaufnahme MIX</t>
   </si>
 </sst>
 </file>
@@ -1762,7 +1765,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="4">
-        <v>-93</v>
+        <v>-95</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -1794,7 +1797,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="4">
-        <v>-6.75</v>
+        <v>-4</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
@@ -1819,7 +1822,7 @@
       </c>
       <c r="B13" s="5">
         <f>SUM(B5:B12)</f>
-        <v>13.300000000000004</v>
+        <v>14.050000000000004</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
@@ -1829,8 +1832,8 @@
       <c r="B14" s="1">
         <v>6</v>
       </c>
-      <c r="C14">
-        <v>5</v>
+      <c r="C14" s="7" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
@@ -1838,7 +1841,7 @@
         <v>14</v>
       </c>
       <c r="B15" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C15">
         <v>6</v>
@@ -1866,7 +1869,7 @@
       </c>
       <c r="B18" s="5">
         <f>-(B16*(B14/100) + B17*(B15/100))</f>
-        <v>-1.1400000000000001</v>
+        <v>-1.02</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
@@ -1875,7 +1878,7 @@
       </c>
       <c r="B19" s="5">
         <f>B13+B18</f>
-        <v>12.160000000000004</v>
+        <v>13.030000000000005</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
@@ -1892,7 +1895,7 @@
       </c>
       <c r="B21" s="5">
         <f>MAX(0, B19-B20)</f>
-        <v>12.160000000000004</v>
+        <v>13.030000000000005</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
@@ -1909,7 +1912,7 @@
       </c>
       <c r="B23" s="5">
         <f>-B21*(B22/100)</f>
-        <v>-5.4720000000000022</v>
+        <v>-5.8635000000000019</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
@@ -1918,7 +1921,7 @@
       </c>
       <c r="B24" s="5">
         <f>B19+B23</f>
-        <v>6.6880000000000015</v>
+        <v>7.1665000000000028</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
@@ -1932,7 +1935,7 @@
         <v>25</v>
       </c>
       <c r="B27" s="4">
-        <v>35.03</v>
+        <v>40.98</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
@@ -1949,7 +1952,7 @@
       </c>
       <c r="B29" s="5">
         <f>B27+B28+B24</f>
-        <v>40.718000000000004</v>
+        <v>47.146500000000003</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
@@ -1958,7 +1961,7 @@
       </c>
       <c r="B30" s="5">
         <f>(B24/B27)*100</f>
-        <v>19.092206679988585</v>
+        <v>17.487798926305523</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
@@ -1973,7 +1976,7 @@
       </c>
       <c r="B33" s="5">
         <f>B24</f>
-        <v>6.6880000000000015</v>
+        <v>7.1665000000000028</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
@@ -1982,7 +1985,7 @@
       </c>
       <c r="B34" s="5">
         <f>-(B10+B11+B12)</f>
-        <v>7</v>
+        <v>4.25</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
@@ -1999,7 +2002,7 @@
       </c>
       <c r="B36" s="5">
         <f>B33+B34+B35</f>
-        <v>15.888000000000002</v>
+        <v>13.616500000000002</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
@@ -2037,7 +2040,7 @@
       </c>
       <c r="B40" s="5">
         <f>B36+B38+B39</f>
-        <v>24.048000000000005</v>
+        <v>21.776500000000006</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.3">
@@ -2107,7 +2110,7 @@
       </c>
       <c r="B51" s="5">
         <f>-B6</f>
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.3">
@@ -2134,7 +2137,7 @@
       </c>
       <c r="B54" s="5">
         <f>-B18</f>
-        <v>1.1400000000000001</v>
+        <v>1.02</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.3">
@@ -2143,7 +2146,7 @@
       </c>
       <c r="B55" s="5">
         <f>-B23</f>
-        <v>5.4720000000000022</v>
+        <v>5.8635000000000019</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.3">
@@ -2159,7 +2162,7 @@
         <v>50</v>
       </c>
       <c r="B57" s="4">
-        <v>17</v>
+        <v>12</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.3">
@@ -2177,7 +2180,7 @@
       </c>
       <c r="B59" s="5">
         <f>SUM(B51:B58)</f>
-        <v>154.71199999999999</v>
+        <v>151.98349999999999</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.3">
@@ -2186,7 +2189,7 @@
       </c>
       <c r="B61" s="5">
         <f>B48-B59</f>
-        <v>3.4080000000000155</v>
+        <v>6.1365000000000123</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.3">
@@ -2203,7 +2206,7 @@
       </c>
       <c r="B63" s="5">
         <f>B61+B62</f>
-        <v>14.668000000000015</v>
+        <v>17.39650000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Minor changes to Excel
</commit_message>
<xml_diff>
--- a/TOPSIM_Planungstool_V8.xlsx
+++ b/TOPSIM_Planungstool_V8.xlsx
@@ -5,18 +5,20 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/96db5acea2ea2686/Hochschule/Sechstes Semester/Business Simulation/Finance Tool/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\FinancePlanningTool_BusinessSimulation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="170" documentId="13_ncr:1_{E0260A73-BE77-4A78-B400-87855D76B609}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DFDC3F65-21B4-4C2E-A002-569A580669EB}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F97B8132-19C7-41E8-9E6A-7064A538CFB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="17496" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Formeln" sheetId="3" r:id="rId1"/>
     <sheet name="Periode 1" sheetId="1" r:id="rId2"/>
     <sheet name="Periode 2" sheetId="2" r:id="rId3"/>
     <sheet name="Periode 3" sheetId="4" r:id="rId4"/>
+    <sheet name="Periode 4" sheetId="6" r:id="rId5"/>
+    <sheet name="Periode 5" sheetId="5" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="71">
   <si>
     <t>Position</t>
   </si>
@@ -252,6 +254,9 @@
   </si>
   <si>
     <t>Im Moment noch 6 aber bei Neuaufnahme MIX</t>
+  </si>
+  <si>
+    <t>Im Moment noch 6 aber bei Neuaufnahme Mix zwischen 5 und 6 (Aufnahmezeitpunkt enscheidend für Zinssatz)</t>
   </si>
 </sst>
 </file>
@@ -395,10 +400,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -687,27 +688,27 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C98663D-40D0-402A-B2D8-812995C4C756}">
   <dimension ref="A1:A5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="39.109375" customWidth="1"/>
+    <col min="1" max="1" width="39.08984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A1" s="9" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="9" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1" ht="58" x14ac:dyDescent="0.35">
       <c r="A4" s="9" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" s="9" t="s">
         <v>67</v>
       </c>
@@ -720,13 +721,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C61"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="65" customWidth="1"/>
     <col min="2" max="2" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -734,13 +735,13 @@
         <v>56</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="2"/>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
@@ -748,7 +749,7 @@
         <v>43000</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
@@ -756,7 +757,7 @@
         <v>3150</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
         <v>4</v>
       </c>
@@ -765,7 +766,7 @@
         <v>135.44999999999999</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
         <v>5</v>
       </c>
@@ -776,7 +777,7 @@
         <v>-38.96</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
         <v>6</v>
       </c>
@@ -784,7 +785,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
         <v>7</v>
       </c>
@@ -792,7 +793,7 @@
         <v>-10</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="s">
         <v>8</v>
       </c>
@@ -800,7 +801,7 @@
         <v>-8</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
         <v>9</v>
       </c>
@@ -808,7 +809,7 @@
         <v>-6.75</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>10</v>
       </c>
@@ -816,7 +817,7 @@
         <v>-0.25</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
         <v>11</v>
       </c>
@@ -824,7 +825,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" s="5" t="s">
         <v>12</v>
       </c>
@@ -833,7 +834,7 @@
         <v>7.4499999999999886</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>13</v>
       </c>
@@ -841,7 +842,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>14</v>
       </c>
@@ -849,7 +850,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="s">
         <v>15</v>
       </c>
@@ -857,7 +858,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" s="4" t="s">
         <v>16</v>
       </c>
@@ -865,7 +866,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" s="5" t="s">
         <v>17</v>
       </c>
@@ -874,7 +875,7 @@
         <v>-1.7100000000000002</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" s="5" t="s">
         <v>18</v>
       </c>
@@ -883,7 +884,7 @@
         <v>5.7399999999999887</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" s="4" t="s">
         <v>19</v>
       </c>
@@ -894,7 +895,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" s="5" t="s">
         <v>20</v>
       </c>
@@ -903,7 +904,7 @@
         <v>5.7399999999999887</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>21</v>
       </c>
@@ -911,7 +912,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" s="5" t="s">
         <v>22</v>
       </c>
@@ -920,7 +921,7 @@
         <v>-2.5829999999999949</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" s="5" t="s">
         <v>23</v>
       </c>
@@ -929,13 +930,13 @@
         <v>3.1569999999999938</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>24</v>
       </c>
       <c r="B26" s="2"/>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" s="4" t="s">
         <v>25</v>
       </c>
@@ -943,7 +944,7 @@
         <v>31.27</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" s="4" t="s">
         <v>26</v>
       </c>
@@ -951,7 +952,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29" s="5" t="s">
         <v>27</v>
       </c>
@@ -960,7 +961,7 @@
         <v>33.426999999999992</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A30" s="5" t="s">
         <v>28</v>
       </c>
@@ -969,13 +970,13 @@
         <v>9.4444610644089941</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
         <v>29</v>
       </c>
       <c r="B32" s="2"/>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A33" s="5" t="s">
         <v>30</v>
       </c>
@@ -984,7 +985,7 @@
         <v>3.1569999999999938</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A34" s="5" t="s">
         <v>31</v>
       </c>
@@ -993,7 +994,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A35" s="4" t="s">
         <v>32</v>
       </c>
@@ -1001,7 +1002,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A36" s="5" t="s">
         <v>33</v>
       </c>
@@ -1010,7 +1011,7 @@
         <v>12.156999999999993</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A37" s="4" t="s">
         <v>34</v>
       </c>
@@ -1022,7 +1023,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A38" s="4" t="s">
         <v>35</v>
       </c>
@@ -1034,7 +1035,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A39" s="5" t="s">
         <v>36</v>
       </c>
@@ -1043,19 +1044,19 @@
         <v>11.626999999999994</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
         <v>37</v>
       </c>
       <c r="B41" s="2"/>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A42" s="6" t="s">
         <v>38</v>
       </c>
       <c r="B42" s="6"/>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A43" s="5" t="s">
         <v>39</v>
       </c>
@@ -1064,7 +1065,7 @@
         <v>108.36</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A44" s="4" t="s">
         <v>40</v>
       </c>
@@ -1072,7 +1073,7 @@
         <v>25.8</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A45" s="4" t="s">
         <v>41</v>
       </c>
@@ -1080,7 +1081,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A46" s="5" t="s">
         <v>42</v>
       </c>
@@ -1089,13 +1090,13 @@
         <v>156.16</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A48" s="6" t="s">
         <v>43</v>
       </c>
       <c r="B48" s="6"/>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A49" s="5" t="s">
         <v>44</v>
       </c>
@@ -1104,7 +1105,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A50" s="5" t="s">
         <v>45</v>
       </c>
@@ -1113,7 +1114,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A51" s="5" t="s">
         <v>46</v>
       </c>
@@ -1122,7 +1123,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A52" s="5" t="s">
         <v>47</v>
       </c>
@@ -1131,7 +1132,7 @@
         <v>1.7100000000000002</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A53" s="5" t="s">
         <v>48</v>
       </c>
@@ -1140,7 +1141,7 @@
         <v>2.5829999999999949</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A54" s="4" t="s">
         <v>49</v>
       </c>
@@ -1148,7 +1149,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A55" s="4" t="s">
         <v>50</v>
       </c>
@@ -1156,7 +1157,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A56" s="5" t="s">
         <v>51</v>
       </c>
@@ -1165,7 +1166,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A57" s="5" t="s">
         <v>52</v>
       </c>
@@ -1174,7 +1175,7 @@
         <v>153.29300000000001</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A59" s="5" t="s">
         <v>53</v>
       </c>
@@ -1183,7 +1184,7 @@
         <v>2.8669999999999902</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A60" s="4" t="s">
         <v>54</v>
       </c>
@@ -1191,7 +1192,7 @@
         <v>11.26</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A61" s="5" t="s">
         <v>55</v>
       </c>
@@ -1209,14 +1210,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3670D53-6421-4BCC-8263-1590D4CFD838}">
   <dimension ref="A1:C63"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="65" customWidth="1"/>
     <col min="2" max="2" width="25" customWidth="1"/>
-    <col min="3" max="3" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1227,13 +1228,13 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="2"/>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
@@ -1241,7 +1242,7 @@
         <v>47000</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
@@ -1249,7 +1250,7 @@
         <v>3200</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
         <v>4</v>
       </c>
@@ -1258,7 +1259,7 @@
         <v>150.4</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
         <v>5</v>
       </c>
@@ -1266,7 +1267,7 @@
         <v>-95</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
         <v>6</v>
       </c>
@@ -1274,7 +1275,7 @@
         <v>-7.1</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
         <v>7</v>
       </c>
@@ -1282,7 +1283,7 @@
         <v>-10</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="s">
         <v>8</v>
       </c>
@@ -1290,7 +1291,7 @@
         <v>-20</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
         <v>9</v>
       </c>
@@ -1298,7 +1299,7 @@
         <v>-6.75</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>10</v>
       </c>
@@ -1306,7 +1307,7 @@
         <v>-0.25</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
         <v>11</v>
       </c>
@@ -1314,7 +1315,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" s="5" t="s">
         <v>12</v>
       </c>
@@ -1323,7 +1324,7 @@
         <v>11.300000000000004</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>13</v>
       </c>
@@ -1331,7 +1332,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>14</v>
       </c>
@@ -1339,7 +1340,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="s">
         <v>15</v>
       </c>
@@ -1347,7 +1348,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" s="4" t="s">
         <v>16</v>
       </c>
@@ -1355,7 +1356,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" s="5" t="s">
         <v>17</v>
       </c>
@@ -1364,7 +1365,7 @@
         <v>-1.31</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" s="5" t="s">
         <v>18</v>
       </c>
@@ -1373,7 +1374,7 @@
         <v>9.9900000000000038</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" s="4" t="s">
         <v>19</v>
       </c>
@@ -1381,7 +1382,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" s="5" t="s">
         <v>20</v>
       </c>
@@ -1390,7 +1391,7 @@
         <v>9.9900000000000038</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>21</v>
       </c>
@@ -1398,7 +1399,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" s="5" t="s">
         <v>22</v>
       </c>
@@ -1407,7 +1408,7 @@
         <v>-4.4955000000000016</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" s="5" t="s">
         <v>23</v>
       </c>
@@ -1416,13 +1417,13 @@
         <v>5.4945000000000022</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>24</v>
       </c>
       <c r="B26" s="2"/>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" s="4" t="s">
         <v>25</v>
       </c>
@@ -1430,7 +1431,7 @@
         <v>35.03</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" s="4" t="s">
         <v>26</v>
       </c>
@@ -1438,7 +1439,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29" s="5" t="s">
         <v>27</v>
       </c>
@@ -1447,7 +1448,7 @@
         <v>39.524500000000003</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30" s="5" t="s">
         <v>28</v>
       </c>
@@ -1456,13 +1457,13 @@
         <v>13.901504130349535</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
         <v>29</v>
       </c>
       <c r="B32" s="2"/>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A33" s="5" t="s">
         <v>30</v>
       </c>
@@ -1471,7 +1472,7 @@
         <v>5.4945000000000022</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A34" s="5" t="s">
         <v>31</v>
       </c>
@@ -1480,7 +1481,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A35" s="4" t="s">
         <v>32</v>
       </c>
@@ -1488,7 +1489,7 @@
         <v>2.2000000000000002</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A36" s="5" t="s">
         <v>33</v>
       </c>
@@ -1497,7 +1498,7 @@
         <v>14.694500000000001</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A37" s="4" t="s">
         <v>64</v>
       </c>
@@ -1505,7 +1506,7 @@
         <v>26.72</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A38" s="4" t="s">
         <v>34</v>
       </c>
@@ -1514,7 +1515,7 @@
         <v>3.360000000000003</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A39" s="4" t="s">
         <v>35</v>
       </c>
@@ -1526,7 +1527,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A40" s="5" t="s">
         <v>36</v>
       </c>
@@ -1535,19 +1536,19 @@
         <v>22.854500000000005</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
         <v>37</v>
       </c>
       <c r="B42" s="2"/>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A43" s="6" t="s">
         <v>38</v>
       </c>
       <c r="B43" s="6"/>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A44" s="5" t="s">
         <v>39</v>
       </c>
@@ -1556,7 +1557,7 @@
         <v>120.32000000000001</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A45" s="4" t="s">
         <v>40</v>
       </c>
@@ -1564,7 +1565,7 @@
         <v>25.8</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A46" s="4" t="s">
         <v>63</v>
       </c>
@@ -1572,7 +1573,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A47" s="4" t="s">
         <v>62</v>
       </c>
@@ -1581,7 +1582,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A48" s="5" t="s">
         <v>42</v>
       </c>
@@ -1590,13 +1591,13 @@
         <v>158.12</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A50" s="6" t="s">
         <v>43</v>
       </c>
       <c r="B50" s="6"/>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A51" s="5" t="s">
         <v>44</v>
       </c>
@@ -1605,7 +1606,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A52" s="5" t="s">
         <v>45</v>
       </c>
@@ -1614,7 +1615,7 @@
         <v>7.1</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A53" s="5" t="s">
         <v>46</v>
       </c>
@@ -1623,7 +1624,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A54" s="5" t="s">
         <v>47</v>
       </c>
@@ -1632,7 +1633,7 @@
         <v>1.31</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A55" s="5" t="s">
         <v>48</v>
       </c>
@@ -1641,7 +1642,7 @@
         <v>4.4955000000000016</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A56" s="4" t="s">
         <v>49</v>
       </c>
@@ -1649,7 +1650,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A57" s="4" t="s">
         <v>50</v>
       </c>
@@ -1657,7 +1658,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A58" s="5" t="s">
         <v>51</v>
       </c>
@@ -1666,7 +1667,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A59" s="5" t="s">
         <v>52</v>
       </c>
@@ -1675,7 +1676,7 @@
         <v>155.90549999999999</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A61" s="5" t="s">
         <v>53</v>
       </c>
@@ -1684,7 +1685,7 @@
         <v>2.2145000000000152</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A62" s="4" t="s">
         <v>54</v>
       </c>
@@ -1692,7 +1693,7 @@
         <v>11.26</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A63" s="5" t="s">
         <v>55</v>
       </c>
@@ -1711,14 +1712,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CDA27C3-61FD-40B5-8531-C2A107CE4E67}">
   <dimension ref="A1:C63"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="65" customWidth="1"/>
     <col min="2" max="2" width="25" customWidth="1"/>
-    <col min="3" max="3" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1729,13 +1730,13 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="2"/>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
@@ -1743,7 +1744,7 @@
         <v>47000</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
@@ -1751,7 +1752,7 @@
         <v>3200</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
         <v>4</v>
       </c>
@@ -1760,7 +1761,7 @@
         <v>150.4</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
         <v>5</v>
       </c>
@@ -1768,7 +1769,7 @@
         <v>-95</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
         <v>6</v>
       </c>
@@ -1776,7 +1777,7 @@
         <v>-7.1</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
         <v>7</v>
       </c>
@@ -1784,7 +1785,7 @@
         <v>-10</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="s">
         <v>8</v>
       </c>
@@ -1792,7 +1793,7 @@
         <v>-20</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
         <v>9</v>
       </c>
@@ -1800,7 +1801,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>10</v>
       </c>
@@ -1808,7 +1809,7 @@
         <v>-0.25</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
         <v>11</v>
       </c>
@@ -1816,7 +1817,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" s="5" t="s">
         <v>12</v>
       </c>
@@ -1825,7 +1826,7 @@
         <v>14.050000000000004</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>13</v>
       </c>
@@ -1836,7 +1837,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>14</v>
       </c>
@@ -1847,7 +1848,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="s">
         <v>15</v>
       </c>
@@ -1855,7 +1856,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" s="4" t="s">
         <v>16</v>
       </c>
@@ -1863,7 +1864,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" s="5" t="s">
         <v>17</v>
       </c>
@@ -1872,7 +1873,7 @@
         <v>-1.02</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" s="5" t="s">
         <v>18</v>
       </c>
@@ -1881,7 +1882,7 @@
         <v>13.030000000000005</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" s="4" t="s">
         <v>19</v>
       </c>
@@ -1889,7 +1890,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" s="5" t="s">
         <v>20</v>
       </c>
@@ -1898,7 +1899,7 @@
         <v>13.030000000000005</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>21</v>
       </c>
@@ -1906,7 +1907,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" s="5" t="s">
         <v>22</v>
       </c>
@@ -1915,7 +1916,7 @@
         <v>-5.8635000000000019</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" s="5" t="s">
         <v>23</v>
       </c>
@@ -1924,13 +1925,13 @@
         <v>7.1665000000000028</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>24</v>
       </c>
       <c r="B26" s="2"/>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" s="4" t="s">
         <v>25</v>
       </c>
@@ -1938,7 +1939,7 @@
         <v>40.98</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" s="4" t="s">
         <v>26</v>
       </c>
@@ -1946,7 +1947,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29" s="5" t="s">
         <v>27</v>
       </c>
@@ -1955,7 +1956,7 @@
         <v>47.146500000000003</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30" s="5" t="s">
         <v>28</v>
       </c>
@@ -1964,13 +1965,13 @@
         <v>17.487798926305523</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
         <v>29</v>
       </c>
       <c r="B32" s="2"/>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A33" s="5" t="s">
         <v>30</v>
       </c>
@@ -1979,7 +1980,7 @@
         <v>7.1665000000000028</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A34" s="5" t="s">
         <v>31</v>
       </c>
@@ -1988,7 +1989,7 @@
         <v>4.25</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A35" s="4" t="s">
         <v>32</v>
       </c>
@@ -1996,7 +1997,7 @@
         <v>2.2000000000000002</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A36" s="5" t="s">
         <v>33</v>
       </c>
@@ -2005,7 +2006,7 @@
         <v>13.616500000000002</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A37" s="4" t="s">
         <v>64</v>
       </c>
@@ -2013,7 +2014,7 @@
         <v>26.72</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A38" s="4" t="s">
         <v>34</v>
       </c>
@@ -2022,7 +2023,7 @@
         <v>3.360000000000003</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A39" s="4" t="s">
         <v>35</v>
       </c>
@@ -2034,7 +2035,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A40" s="5" t="s">
         <v>36</v>
       </c>
@@ -2043,19 +2044,19 @@
         <v>21.776500000000006</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
         <v>37</v>
       </c>
       <c r="B42" s="2"/>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A43" s="6" t="s">
         <v>38</v>
       </c>
       <c r="B43" s="6"/>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A44" s="5" t="s">
         <v>39</v>
       </c>
@@ -2064,7 +2065,7 @@
         <v>120.32000000000001</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A45" s="4" t="s">
         <v>40</v>
       </c>
@@ -2072,7 +2073,7 @@
         <v>25.8</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A46" s="4" t="s">
         <v>63</v>
       </c>
@@ -2080,7 +2081,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A47" s="4" t="s">
         <v>62</v>
       </c>
@@ -2089,7 +2090,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A48" s="5" t="s">
         <v>42</v>
       </c>
@@ -2098,13 +2099,13 @@
         <v>158.12</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A50" s="6" t="s">
         <v>43</v>
       </c>
       <c r="B50" s="6"/>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A51" s="5" t="s">
         <v>44</v>
       </c>
@@ -2113,7 +2114,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A52" s="5" t="s">
         <v>45</v>
       </c>
@@ -2122,7 +2123,7 @@
         <v>7.1</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A53" s="5" t="s">
         <v>46</v>
       </c>
@@ -2131,7 +2132,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A54" s="5" t="s">
         <v>47</v>
       </c>
@@ -2140,7 +2141,7 @@
         <v>1.02</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A55" s="5" t="s">
         <v>48</v>
       </c>
@@ -2149,7 +2150,7 @@
         <v>5.8635000000000019</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A56" s="4" t="s">
         <v>49</v>
       </c>
@@ -2157,7 +2158,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A57" s="4" t="s">
         <v>50</v>
       </c>
@@ -2165,7 +2166,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A58" s="5" t="s">
         <v>51</v>
       </c>
@@ -2174,7 +2175,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A59" s="5" t="s">
         <v>52</v>
       </c>
@@ -2183,7 +2184,7 @@
         <v>151.98349999999999</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A61" s="5" t="s">
         <v>53</v>
       </c>
@@ -2192,7 +2193,7 @@
         <v>6.1365000000000123</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A62" s="4" t="s">
         <v>54</v>
       </c>
@@ -2200,7 +2201,1015 @@
         <v>11.26</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A63" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B63" s="5">
+        <f>B61+B62</f>
+        <v>17.39650000000001</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="4294967293" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0243C56E-5420-43C2-95C0-1BF9EE488613}">
+  <dimension ref="A1:C63"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="65" customWidth="1"/>
+    <col min="2" max="2" width="25" customWidth="1"/>
+    <col min="3" max="3" width="13.1796875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4">
+        <v>47000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4">
+        <v>3200</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="5">
+        <f>B3*B4/1000000</f>
+        <v>150.4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4">
+        <v>-95</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4">
+        <v>-7.1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="4">
+        <v>-10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="4">
+        <v>-20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="4">
+        <v>-4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="1">
+        <v>-0.25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="5">
+        <f>SUM(B5:B12)</f>
+        <v>14.050000000000004</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="1">
+        <v>6</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" s="4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A17" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17" s="4">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A18" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18" s="5">
+        <f>-(B16*(B14/100) + B17*(B15/100))</f>
+        <v>-1.02</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A19" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" s="5">
+        <f>B13+B18</f>
+        <v>13.030000000000005</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A20" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B20" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A21" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" s="5">
+        <f>MAX(0, B19-B20)</f>
+        <v>13.030000000000005</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A22" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22" s="1">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A23" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B23" s="5">
+        <f>-B21*(B22/100)</f>
+        <v>-5.8635000000000019</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A24" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B24" s="5">
+        <f>B19+B23</f>
+        <v>7.1665000000000028</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A26" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B26" s="2"/>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A27" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B27" s="4">
+        <v>40.98</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A28" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B28" s="4">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A29" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B29" s="5">
+        <f>B27+B28+B24</f>
+        <v>47.146500000000003</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A30" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B30" s="5">
+        <f>(B24/B27)*100</f>
+        <v>17.487798926305523</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A32" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B32" s="2"/>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A33" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B33" s="5">
+        <f>B24</f>
+        <v>7.1665000000000028</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A34" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B34" s="5">
+        <f>-(B10+B11+B12)</f>
+        <v>4.25</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A35" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B35" s="4">
+        <v>2.2000000000000002</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A36" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B36" s="5">
+        <f>B33+B34+B35</f>
+        <v>13.616500000000002</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A37" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B37" s="4">
+        <v>26.72</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A38" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B38" s="4">
+        <f>B5*0.2-B37</f>
+        <v>3.360000000000003</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A39" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B39" s="4">
+        <f>4.8</f>
+        <v>4.8</v>
+      </c>
+      <c r="C39" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A40" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B40" s="5">
+        <f>B36+B38+B39</f>
+        <v>21.776500000000006</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A42" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B42" s="2"/>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A43" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B43" s="6"/>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A44" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B44" s="5">
+        <f>B5*0.8</f>
+        <v>120.32000000000001</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A45" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B45" s="4">
+        <v>25.8</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A46" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B46" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A47" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="B47" s="4">
+        <f>B46+B17</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A48" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B48" s="5">
+        <f>B44+B45+B47</f>
+        <v>158.12</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A50" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B50" s="6"/>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A51" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B51" s="5">
+        <f>-B6</f>
+        <v>95</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A52" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="B52" s="5">
+        <f>-B7</f>
+        <v>7.1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A53" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="B53" s="5">
+        <f>-(B8+B9)</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A54" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B54" s="5">
+        <f>-B18</f>
+        <v>1.02</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A55" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B55" s="5">
+        <f>-B23</f>
+        <v>5.8635000000000019</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A56" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B56" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A57" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B57" s="4">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A58" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B58" s="5">
+        <f>-B28</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A59" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B59" s="5">
+        <f>SUM(B51:B58)</f>
+        <v>151.98349999999999</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A61" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B61" s="5">
+        <f>B48-B59</f>
+        <v>6.1365000000000123</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A62" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B62" s="4">
+        <v>11.26</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A63" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B63" s="5">
+        <f>B61+B62</f>
+        <v>17.39650000000001</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="4294967293" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDC343B6-0BFC-4CFB-889F-2B5BEF444628}">
+  <dimension ref="A1:C63"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="65" customWidth="1"/>
+    <col min="2" max="2" width="25" customWidth="1"/>
+    <col min="3" max="3" width="13.1796875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4">
+        <v>47000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4">
+        <v>3200</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="5">
+        <f>B3*B4/1000000</f>
+        <v>150.4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4">
+        <v>-95</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4">
+        <v>-7.1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="4">
+        <v>-10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="4">
+        <v>-20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="4">
+        <v>-4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="1">
+        <v>-0.25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="5">
+        <f>SUM(B5:B12)</f>
+        <v>14.050000000000004</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="1">
+        <v>6</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" s="4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A17" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17" s="4">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A18" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18" s="5">
+        <f>-(B16*(B14/100) + B17*(B15/100))</f>
+        <v>-1.02</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A19" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" s="5">
+        <f>B13+B18</f>
+        <v>13.030000000000005</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A20" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B20" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A21" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" s="5">
+        <f>MAX(0, B19-B20)</f>
+        <v>13.030000000000005</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A22" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22" s="1">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A23" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B23" s="5">
+        <f>-B21*(B22/100)</f>
+        <v>-5.8635000000000019</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A24" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B24" s="5">
+        <f>B19+B23</f>
+        <v>7.1665000000000028</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A26" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B26" s="2"/>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A27" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B27" s="4">
+        <v>40.98</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A28" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B28" s="4">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A29" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B29" s="5">
+        <f>B27+B28+B24</f>
+        <v>47.146500000000003</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A30" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B30" s="5">
+        <f>(B24/B27)*100</f>
+        <v>17.487798926305523</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A32" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B32" s="2"/>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A33" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B33" s="5">
+        <f>B24</f>
+        <v>7.1665000000000028</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A34" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B34" s="5">
+        <f>-(B10+B11+B12)</f>
+        <v>4.25</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A35" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B35" s="4">
+        <v>2.2000000000000002</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A36" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B36" s="5">
+        <f>B33+B34+B35</f>
+        <v>13.616500000000002</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A37" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B37" s="4">
+        <v>26.72</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A38" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B38" s="4">
+        <f>B5*0.2-B37</f>
+        <v>3.360000000000003</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A39" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B39" s="4">
+        <f>4.8</f>
+        <v>4.8</v>
+      </c>
+      <c r="C39" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A40" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B40" s="5">
+        <f>B36+B38+B39</f>
+        <v>21.776500000000006</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A42" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B42" s="2"/>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A43" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B43" s="6"/>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A44" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B44" s="5">
+        <f>B5*0.8</f>
+        <v>120.32000000000001</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A45" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B45" s="4">
+        <v>25.8</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A46" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B46" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A47" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="B47" s="4">
+        <f>B46+B17</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A48" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B48" s="5">
+        <f>B44+B45+B47</f>
+        <v>158.12</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A50" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B50" s="6"/>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A51" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B51" s="5">
+        <f>-B6</f>
+        <v>95</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A52" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="B52" s="5">
+        <f>-B7</f>
+        <v>7.1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A53" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="B53" s="5">
+        <f>-(B8+B9)</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A54" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B54" s="5">
+        <f>-B18</f>
+        <v>1.02</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A55" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B55" s="5">
+        <f>-B23</f>
+        <v>5.8635000000000019</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A56" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B56" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A57" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B57" s="4">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A58" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B58" s="5">
+        <f>-B28</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A59" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B59" s="5">
+        <f>SUM(B51:B58)</f>
+        <v>151.98349999999999</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A61" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B61" s="5">
+        <f>B48-B59</f>
+        <v>6.1365000000000123</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A62" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B62" s="4">
+        <v>11.26</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A63" s="5" t="s">
         <v>55</v>
       </c>

</xml_diff>

<commit_message>
Updated to period 3
</commit_message>
<xml_diff>
--- a/TOPSIM_Planungstool_V8.xlsx
+++ b/TOPSIM_Planungstool_V8.xlsx
@@ -8,17 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/96db5acea2ea2686/Hochschule/Sechstes Semester/Business Simulation/Finance Tool/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="462" documentId="13_ncr:1_{F97B8132-19C7-41E8-9E6A-7064A538CFB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3997C79F-54F7-4B16-890A-9B3B2AFEB21D}"/>
+  <xr:revisionPtr revIDLastSave="628" documentId="13_ncr:1_{F97B8132-19C7-41E8-9E6A-7064A538CFB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EA18D043-09AE-4B82-BA51-F0B4545B132D}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="15552" windowHeight="17376" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="17496" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Formeln" sheetId="3" r:id="rId1"/>
-    <sheet name="Sandbox Periode" sheetId="6" r:id="rId2"/>
-    <sheet name="Periode 1" sheetId="1" r:id="rId3"/>
-    <sheet name="Periode 2" sheetId="2" r:id="rId4"/>
+    <sheet name="Sandbox Periode" sheetId="6" r:id="rId1"/>
+    <sheet name="Periode 1" sheetId="1" r:id="rId2"/>
+    <sheet name="Periode 2 ALT" sheetId="2" r:id="rId3"/>
+    <sheet name="Periode 2 " sheetId="9" r:id="rId4"/>
     <sheet name="Periode 3 ALT" sheetId="4" r:id="rId5"/>
     <sheet name="Periode 3" sheetId="8" r:id="rId6"/>
+    <sheet name="Periode 4" sheetId="10" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="629" uniqueCount="146">
   <si>
     <t>Position</t>
   </si>
@@ -223,14 +224,6 @@
     <t>Kommentar</t>
   </si>
   <si>
-    <t>F&amp;E-Kosten (GuV) = F&amp;E-Mitarbeiter × Gehalt × (1 + PNK%)
-                   + Einstellungs-/Entlassungskosten
-                   + Pensionsrückstellungen (anteilig)
-                   + Gebäude-Abschreibung (5%)
-                   + Ökologie-Budget
-                   + Wertanalyse-Budget</t>
-  </si>
-  <si>
     <t>Kreditaufnahme Summe</t>
   </si>
   <si>
@@ -240,16 +233,6 @@
     <t>Forderungen Vorperiode</t>
   </si>
   <si>
-    <t>Veränderung Vorräte = Δ Materialien + Δ Fertige Erzeugnisse</t>
-  </si>
-  <si>
-    <t>Material-Lager (neu) = Material-Lager (alt) + Einkauf − Verbrauch
-Verbrauch            ≈ Fertigungsmenge × Materialkosten pro Stück / Wertanalyseindex</t>
-  </si>
-  <si>
-    <t>Lager FE (neu) = Lager FE (alt) + Produktion − Absatz   (in Stück, bewertet zu Herstellkosten)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Material: 40500+2843-47000 = -157; Lager: 43500+5858-47000 = 2358 </t>
   </si>
   <si>
@@ -413,13 +396,106 @@
   </si>
   <si>
     <t>Siehe Endbestand Liquiditätsrechnung letze Periode</t>
+  </si>
+  <si>
+    <t>Lagerab oder Zugang</t>
+  </si>
+  <si>
+    <t>Geplante Einkaufsmenge Einsatzstoffe × Staffelpreis</t>
+  </si>
+  <si>
+    <t>3) Fertigungsbericht</t>
+  </si>
+  <si>
+    <t>6) Personal -&gt; Zeile "= Personalendbestand". Basis für P4 vor Fluktuation und Einstellungen</t>
+  </si>
+  <si>
+    <t>Tabelle "Löhne/Gehälter" in NEWS für Gehaltssatz</t>
+  </si>
+  <si>
+    <t> Euer Umweltindex ist gut (96,99). Die Abgabe in P3 lag bei 0,67 MEUR. Du kannst für P4 großzügig ca. 0,60 bis 0,70 MEUR schätzen.</t>
+  </si>
+  <si>
+    <t>Ohne die genauen P3-Kosten zu kennen, solltest du hier sicherheitshalber mit ca. 2,0 MEUR planen, vor allem wenn die Auslastung der Fertigung (P3: 98,6 %) weiterhin hoch bleibt.</t>
+  </si>
+  <si>
+    <t>Plan-Personalbestand: Bestand Vorperiode  - 5 % Fluktuation + Geplante Neueinstellungen</t>
+  </si>
+  <si>
+    <t>Summe aller Löhne/Gehälter (ohne PNK) × 5,0 %</t>
+  </si>
+  <si>
+    <t>Lageranfangsbestand + Geplante Fertigung - Geplanter Absatz; (Lagerendbestand Fertigprodukte × 100 EUR) + (Lagerendbestand Einsatzstoffe × 15 EUR)</t>
+  </si>
+  <si>
+    <t>Geplante Fertigungsmenge × Kosten pro Stück; Kosten pro Stück: Gen 1: ca. 46 EUR / Stück. Gen 2 (aus P3-News): exakt 40 EUR / Stück.</t>
+  </si>
+  <si>
+    <t>(Geplanter Absatz Markt 1 × 25 EUR) + (Geplanter Absatz Markt 2 × 75 EUR)</t>
+  </si>
+  <si>
+    <t>3) Fertigungsbericht, wird nur verändert bei Desinvestition oder Neukauf Anlagen</t>
+  </si>
+  <si>
+    <t>(Fertigungsmenge - Absatzmenge) × Herstellkosten; Lagerabau (+) oder Zugang (-) &lt;- Kosten sind ein positiver Zahlenwert, somit muss es bei Lagerzugang negativ sein (Negative Kosten = Erlöse)</t>
+  </si>
+  <si>
+    <t>Stellschraube (Für Schätzungen oder Tests) (Momentan Lagerbestand)</t>
+  </si>
+  <si>
+    <t>Markt 1: Geplante Absatzmenge (Stück)</t>
+  </si>
+  <si>
+    <t>Markt 1: Geplanter Preis (EUR/Stück)</t>
+  </si>
+  <si>
+    <t>Markt 2: Geplante Absatzmenge (Stück)</t>
+  </si>
+  <si>
+    <t>Markt 2: Geplanter Preis (EUR/Stück)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">20 % Forderungen werden jetzt beglichen, 14) Bilanz -&gt; Aktiva: "Forderungen aus Lieferungen &amp; Leistungen", </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Markt 2 beachten</t>
+    </r>
+  </si>
+  <si>
+    <t>Umrechnung: Dies entspricht ca. 0,7 FCU pro 1 EUR: Hier: 2280/0,7=3257, 14</t>
+  </si>
+  <si>
+    <t>Werbung Markt 2 (MEUR)</t>
+  </si>
+  <si>
+    <t>Fertigung 450, F&amp;E 10, Vertrieb 50</t>
+  </si>
+  <si>
+    <t>Investitionen Umweltanlagen plus neue Anlage</t>
+  </si>
+  <si>
+    <t>Geplante Fertigungsmenge × Einkaufspreis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anzahl Neueinstellungen (gesamt) × 14.000 EUR + Training: Plan-Personalbestand Fertigung × Entscheidungs-Wert </t>
+  </si>
+  <si>
+    <t>Von oben übernehmen, Lagerbestand Vorperiode beachten!! Differenz berechnen</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -457,6 +533,13 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF00B0F0"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -520,7 +603,7 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="2"/>
@@ -536,6 +619,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="2" fillId="5" borderId="0" xfId="4" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="60 % - Akzent1" xfId="3" builtinId="32"/>
@@ -557,6 +641,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -843,39 +931,6 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C98663D-40D0-402A-B2D8-812995C4C756}">
-  <dimension ref="A1:A5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="39.109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:1" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="9" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="9" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A5" s="9" t="s">
-        <v>67</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0243C56E-5420-43C2-95C0-1BF9EE488613}">
   <dimension ref="A1:CB92"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -932,7 +987,7 @@
     </row>
     <row r="6" spans="1:80" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C6"/>
       <c r="D6"/>
@@ -1015,18 +1070,18 @@
     </row>
     <row r="7" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B7" s="4">
         <v>23.65</v>
       </c>
       <c r="C7" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="8" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="B8" s="4">
         <v>2</v>
@@ -1034,7 +1089,7 @@
     </row>
     <row r="9" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="B9" s="4">
         <v>1.1299999999999999</v>
@@ -1042,16 +1097,16 @@
     </row>
     <row r="10" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="B10" s="6"/>
       <c r="C10" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="11" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B11" s="4">
         <v>27.62</v>
@@ -1059,7 +1114,7 @@
     </row>
     <row r="12" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="B12" s="4">
         <v>6.29</v>
@@ -1067,7 +1122,7 @@
     </row>
     <row r="13" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B13" s="4">
         <v>4.51</v>
@@ -1075,7 +1130,7 @@
     </row>
     <row r="14" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B14" s="4">
         <v>3.15</v>
@@ -1083,7 +1138,7 @@
     </row>
     <row r="15" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B15" s="4">
         <v>0.74</v>
@@ -1091,7 +1146,7 @@
     </row>
     <row r="16" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="B16" s="4">
         <v>2.6</v>
@@ -1099,7 +1154,7 @@
     </row>
     <row r="17" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B17" s="4">
         <v>2.12</v>
@@ -1107,7 +1162,7 @@
     </row>
     <row r="18" spans="1:80" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A18" s="6" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C18"/>
       <c r="D18"/>
@@ -1190,18 +1245,18 @@
     </row>
     <row r="19" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B19" s="4">
         <v>40</v>
       </c>
       <c r="C19" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
     </row>
     <row r="20" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B20" s="5">
         <f>ROUNDUP(SUM(B11:B15)*(B19/100),2)</f>
@@ -1210,7 +1265,7 @@
     </row>
     <row r="21" spans="1:80" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C21"/>
       <c r="D21"/>
@@ -1293,7 +1348,7 @@
     </row>
     <row r="22" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B22" s="4">
         <v>5.5</v>
@@ -1301,7 +1356,7 @@
     </row>
     <row r="23" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="B23" s="4">
         <v>0.65</v>
@@ -1317,7 +1372,7 @@
     </row>
     <row r="25" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="B25" s="5">
         <f>SUM(B22:B24)</f>
@@ -1326,7 +1381,7 @@
     </row>
     <row r="26" spans="1:80" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A26" s="6" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="B26" s="6"/>
       <c r="C26"/>
@@ -1410,7 +1465,7 @@
     </row>
     <row r="27" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B27" s="4">
         <v>3.25</v>
@@ -1418,7 +1473,7 @@
     </row>
     <row r="28" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B28" s="4">
         <v>7</v>
@@ -1426,7 +1481,7 @@
     </row>
     <row r="29" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B29" s="4">
         <v>2</v>
@@ -1434,7 +1489,7 @@
     </row>
     <row r="30" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="B30" s="4">
         <v>0.8</v>
@@ -1442,7 +1497,7 @@
     </row>
     <row r="31" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="B31" s="4">
         <v>1.78</v>
@@ -1450,7 +1505,7 @@
     </row>
     <row r="32" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="B32" s="4">
         <v>0.48</v>
@@ -1458,13 +1513,13 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" s="6" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B33" s="6"/>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="B34" s="4">
         <v>8</v>
@@ -1472,7 +1527,7 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="B35" s="4">
         <v>3.5</v>
@@ -1480,7 +1535,7 @@
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="B36" s="4">
         <v>2.5</v>
@@ -1488,7 +1543,7 @@
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="B37" s="4">
         <v>1</v>
@@ -1496,7 +1551,7 @@
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="B38" s="1">
         <v>3.88</v>
@@ -1504,7 +1559,7 @@
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" s="5" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B39" s="5">
         <f>-SUM(B7:B9,(B11:B17),B20,B25,(B27:B32),B34:B38)</f>
@@ -1513,13 +1568,13 @@
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" s="6" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="B40" s="6"/>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" s="5" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="B41" s="5">
         <f>ROUNDUP(SUM(B5,B39),2)</f>
@@ -1534,7 +1589,7 @@
         <v>6</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.3">
@@ -1545,7 +1600,7 @@
         <v>6.5</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.3">
@@ -1558,7 +1613,7 @@
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45" s="4" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B45" s="4">
         <v>12</v>
@@ -1691,7 +1746,7 @@
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A63" s="5" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B63" s="5">
         <f>B17</f>
@@ -1709,7 +1764,7 @@
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A65" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B65" s="4">
         <v>26.72</v>
@@ -1733,7 +1788,7 @@
         <v>4.5599999999999996</v>
       </c>
       <c r="C67" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.3">
@@ -1774,12 +1829,12 @@
         <v>26.72</v>
       </c>
       <c r="C73" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A74" s="4" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="B74" s="4">
         <v>0</v>
@@ -1787,7 +1842,7 @@
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A75" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B75" s="5">
         <f>B74+B45</f>
@@ -1811,18 +1866,18 @@
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A78" s="4" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="B78" s="4">
         <v>22.96</v>
       </c>
       <c r="C78" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A79" s="5" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="B79" s="5">
         <f>B8</f>
@@ -1831,7 +1886,7 @@
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A80" s="5" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B80" s="5">
         <f>SUM(B78:B79)</f>
@@ -1840,7 +1895,7 @@
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A81" s="5" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="B81" s="5">
         <f>SUM(B11:B16,B20)</f>
@@ -1849,7 +1904,7 @@
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A82" s="5" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="B82" s="5">
         <f>SUM(B27:B32,B34:B37,B9)</f>
@@ -1882,7 +1937,7 @@
         <v>2.5</v>
       </c>
       <c r="C85" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.3">
@@ -1893,7 +1948,7 @@
         <v>17</v>
       </c>
       <c r="C86" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.3">
@@ -1916,7 +1971,7 @@
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A89" s="6" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="B89" s="6"/>
     </row>
@@ -1937,7 +1992,7 @@
         <v>10.1</v>
       </c>
       <c r="C91" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.3">
@@ -1958,7 +2013,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C61"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2447,7 +2502,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3670D53-6421-4BCC-8263-1590D4CFD838}">
   <dimension ref="A1:C63"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2740,7 +2795,7 @@
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B37" s="4">
         <v>26.72</v>
@@ -2764,7 +2819,7 @@
         <v>4.8</v>
       </c>
       <c r="C39" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
@@ -2807,7 +2862,7 @@
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B46" s="4">
         <v>0</v>
@@ -2815,7 +2870,7 @@
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A47" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B47" s="4">
         <f>B46+B17</f>
@@ -2949,521 +3004,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CDA27C3-61FD-40B5-8531-C2A107CE4E67}">
-  <dimension ref="A1:C62"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="65" customWidth="1"/>
-    <col min="2" max="2" width="25" customWidth="1"/>
-    <col min="3" max="3" width="13.21875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2"/>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" s="4">
-        <v>47000</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="4">
-        <v>3200</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" s="5">
-        <f>B3*B4/1000000</f>
-        <v>150.4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6" s="4">
-        <v>-95</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7" s="4">
-        <v>-7.1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8" s="4">
-        <v>-10</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9" s="4">
-        <v>-20</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B10" s="4">
-        <v>-4</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B11" s="1">
-        <v>-0.25</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B12" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B13" s="5">
-        <f>SUM(B5:B12)</f>
-        <v>14.050000000000004</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B14" s="1">
-        <v>6</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B15" s="1">
-        <v>6</v>
-      </c>
-      <c r="C15">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B16" s="4">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A17" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B17" s="4">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="B18" s="5">
-        <f>-(B16*(B14/100) + B17*(B15/100))</f>
-        <v>-1.02</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A19" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B19" s="5">
-        <f>B13+B18</f>
-        <v>13.030000000000005</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A20" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B20" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A21" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B21" s="5">
-        <f>MAX(0, B19-B20)</f>
-        <v>13.030000000000005</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A22" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B22" s="1">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A23" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="B23" s="5">
-        <f>-B21*(B22/100)</f>
-        <v>-5.8635000000000019</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A24" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="B24" s="5">
-        <f>B19+B23</f>
-        <v>7.1665000000000028</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A26" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B26" s="2"/>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A27" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B27" s="4">
-        <v>40.98</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A28" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B28" s="4">
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A29" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="B29" s="5">
-        <f>B27+B28+B24</f>
-        <v>47.146500000000003</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A30" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="B30" s="5">
-        <f>(B24/B27)*100</f>
-        <v>17.487798926305523</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A32" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="B32" s="2"/>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A33" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="B33" s="5">
-        <f>B24</f>
-        <v>7.1665000000000028</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A34" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="B34" s="5">
-        <f>-(B10+B11+B12)</f>
-        <v>4.25</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A35" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="B35" s="4">
-        <v>2.2000000000000002</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A36" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="B36" s="5">
-        <f>B33+B34+B35</f>
-        <v>13.616500000000002</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A37" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="B37" s="4">
-        <v>26.72</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A38" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="B38" s="4">
-        <f>B5*0.2-B37</f>
-        <v>3.360000000000003</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A39" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="B39" s="4">
-        <f>4.8</f>
-        <v>4.8</v>
-      </c>
-      <c r="C39" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A40" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="B40" s="5">
-        <f>B36+B38+B39</f>
-        <v>21.776500000000006</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A42" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B42" s="2"/>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A43" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B43" s="6"/>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A44" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="B44" s="5">
-        <f>B5*0.8</f>
-        <v>120.32000000000001</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A45" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="B45" s="4">
-        <v>25.8</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A46" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="B46" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A47" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="B47" s="4">
-        <f>B46+B17</f>
-        <v>12</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A48" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="B48" s="5">
-        <f>B44+B45+B47</f>
-        <v>158.12</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A49" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="B49" s="6"/>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A50" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="B50" s="5">
-        <f>-B6</f>
-        <v>95</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A51" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="B51" s="5">
-        <f>-B7</f>
-        <v>7.1</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A52" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="B52" s="5">
-        <f>-(B8+B9)</f>
-        <v>30</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A53" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="B53" s="5">
-        <f>-B18</f>
-        <v>1.02</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A54" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="B54" s="5">
-        <f>-B23</f>
-        <v>5.8635000000000019</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A55" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="B55" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A56" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="B56" s="4">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A57" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="B57" s="5">
-        <f>-B28</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A58" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="B58" s="5">
-        <f>SUM(B50:B57)</f>
-        <v>151.98349999999999</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A59" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="B59" s="6"/>
-    </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A60" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="B60" s="5">
-        <f>B48-B58</f>
-        <v>6.1365000000000123</v>
-      </c>
-    </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A61" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="B61" s="4">
-        <v>11.26</v>
-      </c>
-    </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A62" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="B62" s="5">
-        <f>B60+B61</f>
-        <v>17.39650000000001</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="4294967293" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A2DB656-79A9-4C5A-8517-D8CA2ED228B1}">
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30356088-4FC0-428D-AFAB-E77B08EE9E82}">
   <dimension ref="A1:CB92"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -3519,7 +3061,7 @@
     </row>
     <row r="6" spans="1:80" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C6"/>
       <c r="D6"/>
@@ -3602,18 +3144,18 @@
     </row>
     <row r="7" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B7" s="4">
         <v>23.65</v>
       </c>
       <c r="C7" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="8" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="B8" s="4">
         <v>2</v>
@@ -3621,7 +3163,7 @@
     </row>
     <row r="9" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="B9" s="4">
         <v>1.1299999999999999</v>
@@ -3629,16 +3171,16 @@
     </row>
     <row r="10" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="B10" s="6"/>
       <c r="C10" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="11" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B11" s="4">
         <v>27.62</v>
@@ -3646,7 +3188,7 @@
     </row>
     <row r="12" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="B12" s="4">
         <v>6.29</v>
@@ -3654,7 +3196,7 @@
     </row>
     <row r="13" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B13" s="4">
         <v>4.51</v>
@@ -3662,7 +3204,7 @@
     </row>
     <row r="14" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B14" s="4">
         <v>3.15</v>
@@ -3670,7 +3212,7 @@
     </row>
     <row r="15" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B15" s="4">
         <v>0.74</v>
@@ -3678,7 +3220,7 @@
     </row>
     <row r="16" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="B16" s="4">
         <v>2.6</v>
@@ -3686,7 +3228,7 @@
     </row>
     <row r="17" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B17" s="4">
         <v>2.12</v>
@@ -3694,7 +3236,7 @@
     </row>
     <row r="18" spans="1:80" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A18" s="6" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C18"/>
       <c r="D18"/>
@@ -3777,18 +3319,18 @@
     </row>
     <row r="19" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B19" s="4">
         <v>40</v>
       </c>
       <c r="C19" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
     </row>
     <row r="20" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B20" s="5">
         <f>ROUNDUP(SUM(B11:B15)*(B19/100),2)</f>
@@ -3797,7 +3339,7 @@
     </row>
     <row r="21" spans="1:80" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C21"/>
       <c r="D21"/>
@@ -3880,7 +3422,7 @@
     </row>
     <row r="22" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B22" s="4">
         <v>5.5</v>
@@ -3888,7 +3430,7 @@
     </row>
     <row r="23" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="B23" s="4">
         <v>0.65</v>
@@ -3904,7 +3446,7 @@
     </row>
     <row r="25" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="B25" s="5">
         <f>SUM(B22:B24)</f>
@@ -3913,7 +3455,7 @@
     </row>
     <row r="26" spans="1:80" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A26" s="6" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="B26" s="6"/>
       <c r="C26"/>
@@ -3997,7 +3539,7 @@
     </row>
     <row r="27" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B27" s="4">
         <v>3.25</v>
@@ -4005,7 +3547,7 @@
     </row>
     <row r="28" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B28" s="4">
         <v>7</v>
@@ -4013,7 +3555,7 @@
     </row>
     <row r="29" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B29" s="4">
         <v>2</v>
@@ -4021,7 +3563,7 @@
     </row>
     <row r="30" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="B30" s="4">
         <v>0.8</v>
@@ -4029,7 +3571,7 @@
     </row>
     <row r="31" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="B31" s="4">
         <v>1.78</v>
@@ -4037,7 +3579,7 @@
     </row>
     <row r="32" spans="1:80" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="B32" s="4">
         <v>0.48</v>
@@ -4045,13 +3587,13 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" s="6" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B33" s="6"/>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="B34" s="4">
         <v>8</v>
@@ -4059,7 +3601,7 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="B35" s="4">
         <v>3.5</v>
@@ -4067,7 +3609,7 @@
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="B36" s="4">
         <v>2.5</v>
@@ -4075,7 +3617,7 @@
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="B37" s="4">
         <v>1</v>
@@ -4083,15 +3625,18 @@
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="B38" s="1">
         <v>3.88</v>
       </c>
+      <c r="C38" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" s="5" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B39" s="5">
         <f>-SUM(B7:B9,(B11:B17),B20,B25,(B27:B32),B34:B38)</f>
@@ -4100,13 +3645,13 @@
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" s="6" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="B40" s="6"/>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" s="5" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="B41" s="5">
         <f>ROUNDUP(SUM(B5,B39),2)</f>
@@ -4121,7 +3666,7 @@
         <v>6</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.3">
@@ -4132,7 +3677,7 @@
         <v>6.5</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.3">
@@ -4145,7 +3690,7 @@
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45" s="4" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B45" s="4">
         <v>12</v>
@@ -4278,7 +3823,7 @@
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A63" s="5" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B63" s="5">
         <f>B17</f>
@@ -4296,7 +3841,7 @@
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A65" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B65" s="4">
         <v>26.72</v>
@@ -4320,7 +3865,7 @@
         <v>4.5599999999999996</v>
       </c>
       <c r="C67" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.3">
@@ -4361,12 +3906,12 @@
         <v>26.72</v>
       </c>
       <c r="C73" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A74" s="4" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="B74" s="4">
         <v>0</v>
@@ -4374,7 +3919,7 @@
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A75" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B75" s="5">
         <f>B74+B45</f>
@@ -4398,18 +3943,18 @@
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A78" s="4" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="B78" s="4">
         <v>22.96</v>
       </c>
       <c r="C78" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A79" s="5" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="B79" s="5">
         <f>B8</f>
@@ -4418,7 +3963,7 @@
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A80" s="5" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B80" s="5">
         <f>SUM(B78:B79)</f>
@@ -4427,7 +3972,7 @@
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A81" s="5" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="B81" s="5">
         <f>SUM(B11:B16,B20)</f>
@@ -4436,7 +3981,7 @@
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A82" s="5" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="B82" s="5">
         <f>SUM(B27:B32,B34:B37,B9)</f>
@@ -4469,7 +4014,7 @@
         <v>2.5</v>
       </c>
       <c r="C85" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.3">
@@ -4480,7 +4025,7 @@
         <v>17</v>
       </c>
       <c r="C86" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.3">
@@ -4503,7 +4048,7 @@
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A89" s="6" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="B89" s="6"/>
     </row>
@@ -4524,7 +4069,7 @@
         <v>10.1</v>
       </c>
       <c r="C91" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.3">
@@ -4534,6 +4079,2846 @@
       <c r="B92" s="5">
         <f>B90+B91</f>
         <v>19.344560000000037</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="4294967293" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CDA27C3-61FD-40B5-8531-C2A107CE4E67}">
+  <dimension ref="A1:C62"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="65" customWidth="1"/>
+    <col min="2" max="2" width="25" customWidth="1"/>
+    <col min="3" max="3" width="13.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4">
+        <v>47000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4">
+        <v>3200</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="5">
+        <f>B3*B4/1000000</f>
+        <v>150.4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4">
+        <v>-95</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4">
+        <v>-7.1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="4">
+        <v>-10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="4">
+        <v>-20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="4">
+        <v>-4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="1">
+        <v>-0.25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="5">
+        <f>SUM(B5:B12)</f>
+        <v>14.050000000000004</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="1">
+        <v>6</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" s="1">
+        <v>6</v>
+      </c>
+      <c r="C15">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" s="4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17" s="4">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18" s="5">
+        <f>-(B16*(B14/100) + B17*(B15/100))</f>
+        <v>-1.02</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" s="5">
+        <f>B13+B18</f>
+        <v>13.030000000000005</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B20" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" s="5">
+        <f>MAX(0, B19-B20)</f>
+        <v>13.030000000000005</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A22" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22" s="1">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A23" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B23" s="5">
+        <f>-B21*(B22/100)</f>
+        <v>-5.8635000000000019</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A24" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B24" s="5">
+        <f>B19+B23</f>
+        <v>7.1665000000000028</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A26" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B26" s="2"/>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A27" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B27" s="4">
+        <v>40.98</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A28" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B28" s="4">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A29" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B29" s="5">
+        <f>B27+B28+B24</f>
+        <v>47.146500000000003</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A30" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B30" s="5">
+        <f>(B24/B27)*100</f>
+        <v>17.487798926305523</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A32" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B32" s="2"/>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B33" s="5">
+        <f>B24</f>
+        <v>7.1665000000000028</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B34" s="5">
+        <f>-(B10+B11+B12)</f>
+        <v>4.25</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B35" s="4">
+        <v>2.2000000000000002</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B36" s="5">
+        <f>B33+B34+B35</f>
+        <v>13.616500000000002</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B37" s="4">
+        <v>26.72</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A38" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B38" s="4">
+        <f>B5*0.2-B37</f>
+        <v>3.360000000000003</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B39" s="4">
+        <f>4.8</f>
+        <v>4.8</v>
+      </c>
+      <c r="C39" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A40" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B40" s="5">
+        <f>B36+B38+B39</f>
+        <v>21.776500000000006</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A42" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B42" s="2"/>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A43" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B43" s="6"/>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A44" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B44" s="5">
+        <f>B5*0.8</f>
+        <v>120.32000000000001</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A45" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B45" s="4">
+        <v>25.8</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A46" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="B46" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A47" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B47" s="4">
+        <f>B46+B17</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A48" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B48" s="5">
+        <f>B44+B45+B47</f>
+        <v>158.12</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A49" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B49" s="6"/>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A50" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B50" s="5">
+        <f>-B6</f>
+        <v>95</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A51" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="B51" s="5">
+        <f>-B7</f>
+        <v>7.1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A52" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="B52" s="5">
+        <f>-(B8+B9)</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A53" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B53" s="5">
+        <f>-B18</f>
+        <v>1.02</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A54" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B54" s="5">
+        <f>-B23</f>
+        <v>5.8635000000000019</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A55" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B55" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A56" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B56" s="4">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A57" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B57" s="5">
+        <f>-B28</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A58" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B58" s="5">
+        <f>SUM(B50:B57)</f>
+        <v>151.98349999999999</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A59" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B59" s="6"/>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A60" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B60" s="5">
+        <f>B48-B58</f>
+        <v>6.1365000000000123</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A61" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B61" s="4">
+        <v>11.26</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A62" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B62" s="5">
+        <f>B60+B61</f>
+        <v>17.39650000000001</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="4294967293" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A2DB656-79A9-4C5A-8517-D8CA2ED228B1}">
+  <dimension ref="A1:CB95"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="57.33203125" customWidth="1"/>
+    <col min="2" max="2" width="25" customWidth="1"/>
+    <col min="3" max="3" width="153.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+    </row>
+    <row r="2" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2"/>
+    </row>
+    <row r="3" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="B3" s="10">
+        <v>55000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B4" s="4">
+        <v>3170</v>
+      </c>
+    </row>
+    <row r="5" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="B5" s="4">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="B6" s="4">
+        <v>3257.14</v>
+      </c>
+      <c r="C6" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="7" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A7" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" s="5">
+        <f>(B3*B4/1000000)+(B5*B6/1000000)</f>
+        <v>193.89284000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:80" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="C8"/>
+      <c r="D8"/>
+      <c r="E8"/>
+      <c r="F8"/>
+      <c r="G8"/>
+      <c r="H8"/>
+      <c r="I8"/>
+      <c r="J8"/>
+      <c r="K8"/>
+      <c r="L8"/>
+      <c r="M8"/>
+      <c r="N8"/>
+      <c r="O8"/>
+      <c r="P8"/>
+      <c r="Q8"/>
+      <c r="R8"/>
+      <c r="S8"/>
+      <c r="T8"/>
+      <c r="U8"/>
+      <c r="V8"/>
+      <c r="W8"/>
+      <c r="X8"/>
+      <c r="Y8"/>
+      <c r="Z8"/>
+      <c r="AA8"/>
+      <c r="AB8"/>
+      <c r="AC8"/>
+      <c r="AD8"/>
+      <c r="AE8"/>
+      <c r="AF8"/>
+      <c r="AG8"/>
+      <c r="AH8"/>
+      <c r="AI8"/>
+      <c r="AJ8"/>
+      <c r="AK8"/>
+      <c r="AL8"/>
+      <c r="AM8"/>
+      <c r="AN8"/>
+      <c r="AO8"/>
+      <c r="AP8"/>
+      <c r="AQ8"/>
+      <c r="AR8"/>
+      <c r="AS8"/>
+      <c r="AT8"/>
+      <c r="AU8"/>
+      <c r="AV8"/>
+      <c r="AW8"/>
+      <c r="AX8"/>
+      <c r="AY8"/>
+      <c r="AZ8"/>
+      <c r="BA8"/>
+      <c r="BB8"/>
+      <c r="BC8"/>
+      <c r="BD8"/>
+      <c r="BE8"/>
+      <c r="BF8"/>
+      <c r="BG8"/>
+      <c r="BH8"/>
+      <c r="BI8"/>
+      <c r="BJ8"/>
+      <c r="BK8"/>
+      <c r="BL8"/>
+      <c r="BM8"/>
+      <c r="BN8"/>
+      <c r="BO8"/>
+      <c r="BP8"/>
+      <c r="BQ8"/>
+      <c r="BR8"/>
+      <c r="BS8"/>
+      <c r="BT8"/>
+      <c r="BU8"/>
+      <c r="BV8"/>
+      <c r="BW8"/>
+      <c r="BX8"/>
+      <c r="BY8"/>
+      <c r="BZ8"/>
+      <c r="CA8"/>
+      <c r="CB8"/>
+    </row>
+    <row r="9" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A9" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B9" s="4">
+        <f>(66000*350)/1000000</f>
+        <v>23.1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="10" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A10" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B10" s="4">
+        <f>(66000*40)/1000000</f>
+        <v>2.64</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="11" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A11" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B11" s="4">
+        <f>(B3*25+B5*75)/1000000</f>
+        <v>1.825</v>
+      </c>
+      <c r="C11" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="12" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A12" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B12" s="6"/>
+      <c r="C12" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="13" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A13" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="B13" s="4">
+        <f>(((975-(975*0.05))+450)*32000)/1000000</f>
+        <v>44.04</v>
+      </c>
+      <c r="C13" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="14" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A14" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B14" s="4">
+        <f>(300*30000)/1000000</f>
+        <v>9</v>
+      </c>
+      <c r="C14" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="15" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A15" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B15" s="4">
+        <f>(((120-(120*0.05))+50)*43000)/1000000</f>
+        <v>7.0519999999999996</v>
+      </c>
+      <c r="C15" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="16" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A16" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B16" s="4">
+        <f>(((120-(120*0.05))+10)*47000)/1000000</f>
+        <v>5.8280000000000003</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="17" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A17" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="B17" s="4">
+        <f>(34*32000)/1000000</f>
+        <v>1.0880000000000001</v>
+      </c>
+    </row>
+    <row r="18" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A18" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B18" s="4">
+        <f>(510*14000+1377*1200)/1000000</f>
+        <v>8.7924000000000007</v>
+      </c>
+      <c r="C18" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="19" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A19" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="B19" s="5">
+        <f>SUM(B13:B18)*0.05</f>
+        <v>3.7900200000000002</v>
+      </c>
+      <c r="C19" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="20" spans="1:80" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="C20"/>
+      <c r="D20"/>
+      <c r="E20"/>
+      <c r="F20"/>
+      <c r="G20"/>
+      <c r="H20"/>
+      <c r="I20"/>
+      <c r="J20"/>
+      <c r="K20"/>
+      <c r="L20"/>
+      <c r="M20"/>
+      <c r="N20"/>
+      <c r="O20"/>
+      <c r="P20"/>
+      <c r="Q20"/>
+      <c r="R20"/>
+      <c r="S20"/>
+      <c r="T20"/>
+      <c r="U20"/>
+      <c r="V20"/>
+      <c r="W20"/>
+      <c r="X20"/>
+      <c r="Y20"/>
+      <c r="Z20"/>
+      <c r="AA20"/>
+      <c r="AB20"/>
+      <c r="AC20"/>
+      <c r="AD20"/>
+      <c r="AE20"/>
+      <c r="AF20"/>
+      <c r="AG20"/>
+      <c r="AH20"/>
+      <c r="AI20"/>
+      <c r="AJ20"/>
+      <c r="AK20"/>
+      <c r="AL20"/>
+      <c r="AM20"/>
+      <c r="AN20"/>
+      <c r="AO20"/>
+      <c r="AP20"/>
+      <c r="AQ20"/>
+      <c r="AR20"/>
+      <c r="AS20"/>
+      <c r="AT20"/>
+      <c r="AU20"/>
+      <c r="AV20"/>
+      <c r="AW20"/>
+      <c r="AX20"/>
+      <c r="AY20"/>
+      <c r="AZ20"/>
+      <c r="BA20"/>
+      <c r="BB20"/>
+      <c r="BC20"/>
+      <c r="BD20"/>
+      <c r="BE20"/>
+      <c r="BF20"/>
+      <c r="BG20"/>
+      <c r="BH20"/>
+      <c r="BI20"/>
+      <c r="BJ20"/>
+      <c r="BK20"/>
+      <c r="BL20"/>
+      <c r="BM20"/>
+      <c r="BN20"/>
+      <c r="BO20"/>
+      <c r="BP20"/>
+      <c r="BQ20"/>
+      <c r="BR20"/>
+      <c r="BS20"/>
+      <c r="BT20"/>
+      <c r="BU20"/>
+      <c r="BV20"/>
+      <c r="BW20"/>
+      <c r="BX20"/>
+      <c r="BY20"/>
+      <c r="BZ20"/>
+      <c r="CA20"/>
+      <c r="CB20"/>
+    </row>
+    <row r="21" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A21" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="B21" s="4">
+        <v>40</v>
+      </c>
+      <c r="C21" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="22" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A22" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="B22" s="5">
+        <f>ROUNDUP(SUM(B13:B17)*(B21/100),2)</f>
+        <v>26.810000000000002</v>
+      </c>
+    </row>
+    <row r="23" spans="1:80" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C23"/>
+      <c r="D23"/>
+      <c r="E23"/>
+      <c r="F23"/>
+      <c r="G23"/>
+      <c r="H23"/>
+      <c r="I23"/>
+      <c r="J23"/>
+      <c r="K23"/>
+      <c r="L23"/>
+      <c r="M23"/>
+      <c r="N23"/>
+      <c r="O23"/>
+      <c r="P23"/>
+      <c r="Q23"/>
+      <c r="R23"/>
+      <c r="S23"/>
+      <c r="T23"/>
+      <c r="U23"/>
+      <c r="V23"/>
+      <c r="W23"/>
+      <c r="X23"/>
+      <c r="Y23"/>
+      <c r="Z23"/>
+      <c r="AA23"/>
+      <c r="AB23"/>
+      <c r="AC23"/>
+      <c r="AD23"/>
+      <c r="AE23"/>
+      <c r="AF23"/>
+      <c r="AG23"/>
+      <c r="AH23"/>
+      <c r="AI23"/>
+      <c r="AJ23"/>
+      <c r="AK23"/>
+      <c r="AL23"/>
+      <c r="AM23"/>
+      <c r="AN23"/>
+      <c r="AO23"/>
+      <c r="AP23"/>
+      <c r="AQ23"/>
+      <c r="AR23"/>
+      <c r="AS23"/>
+      <c r="AT23"/>
+      <c r="AU23"/>
+      <c r="AV23"/>
+      <c r="AW23"/>
+      <c r="AX23"/>
+      <c r="AY23"/>
+      <c r="AZ23"/>
+      <c r="BA23"/>
+      <c r="BB23"/>
+      <c r="BC23"/>
+      <c r="BD23"/>
+      <c r="BE23"/>
+      <c r="BF23"/>
+      <c r="BG23"/>
+      <c r="BH23"/>
+      <c r="BI23"/>
+      <c r="BJ23"/>
+      <c r="BK23"/>
+      <c r="BL23"/>
+      <c r="BM23"/>
+      <c r="BN23"/>
+      <c r="BO23"/>
+      <c r="BP23"/>
+      <c r="BQ23"/>
+      <c r="BR23"/>
+      <c r="BS23"/>
+      <c r="BT23"/>
+      <c r="BU23"/>
+      <c r="BV23"/>
+      <c r="BW23"/>
+      <c r="BX23"/>
+      <c r="BY23"/>
+      <c r="BZ23"/>
+      <c r="CA23"/>
+      <c r="CB23"/>
+    </row>
+    <row r="24" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A24" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B24" s="4">
+        <v>4</v>
+      </c>
+      <c r="C24" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="25" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A25" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B25" s="4">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="26" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A26" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B26" s="1">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A27" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="B27" s="5">
+        <f>SUM(B24:B26)</f>
+        <v>5.05</v>
+      </c>
+    </row>
+    <row r="28" spans="1:80" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="B28" s="6"/>
+      <c r="C28"/>
+      <c r="D28"/>
+      <c r="E28"/>
+      <c r="F28"/>
+      <c r="G28"/>
+      <c r="H28"/>
+      <c r="I28"/>
+      <c r="J28"/>
+      <c r="K28"/>
+      <c r="L28"/>
+      <c r="M28"/>
+      <c r="N28"/>
+      <c r="O28"/>
+      <c r="P28"/>
+      <c r="Q28"/>
+      <c r="R28"/>
+      <c r="S28"/>
+      <c r="T28"/>
+      <c r="U28"/>
+      <c r="V28"/>
+      <c r="W28"/>
+      <c r="X28"/>
+      <c r="Y28"/>
+      <c r="Z28"/>
+      <c r="AA28"/>
+      <c r="AB28"/>
+      <c r="AC28"/>
+      <c r="AD28"/>
+      <c r="AE28"/>
+      <c r="AF28"/>
+      <c r="AG28"/>
+      <c r="AH28"/>
+      <c r="AI28"/>
+      <c r="AJ28"/>
+      <c r="AK28"/>
+      <c r="AL28"/>
+      <c r="AM28"/>
+      <c r="AN28"/>
+      <c r="AO28"/>
+      <c r="AP28"/>
+      <c r="AQ28"/>
+      <c r="AR28"/>
+      <c r="AS28"/>
+      <c r="AT28"/>
+      <c r="AU28"/>
+      <c r="AV28"/>
+      <c r="AW28"/>
+      <c r="AX28"/>
+      <c r="AY28"/>
+      <c r="AZ28"/>
+      <c r="BA28"/>
+      <c r="BB28"/>
+      <c r="BC28"/>
+      <c r="BD28"/>
+      <c r="BE28"/>
+      <c r="BF28"/>
+      <c r="BG28"/>
+      <c r="BH28"/>
+      <c r="BI28"/>
+      <c r="BJ28"/>
+      <c r="BK28"/>
+      <c r="BL28"/>
+      <c r="BM28"/>
+      <c r="BN28"/>
+      <c r="BO28"/>
+      <c r="BP28"/>
+      <c r="BQ28"/>
+      <c r="BR28"/>
+      <c r="BS28"/>
+      <c r="BT28"/>
+      <c r="BU28"/>
+      <c r="BV28"/>
+      <c r="BW28"/>
+      <c r="BX28"/>
+      <c r="BY28"/>
+      <c r="BZ28"/>
+      <c r="CA28"/>
+      <c r="CB28"/>
+    </row>
+    <row r="29" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A29" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="B29" s="4">
+        <v>4.75</v>
+      </c>
+      <c r="C29" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="30" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A30" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="B30" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="31" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A31" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B31" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A32" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B32" s="4">
+        <v>0.7</v>
+      </c>
+      <c r="C32" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="B33" s="4">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B34" s="4">
+        <f>(5000*100+4000*15)/1000000</f>
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="C34" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="B35" s="6"/>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B36" s="4">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="B37" s="4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A38" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B38" s="4">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="B39" s="4">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A40" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B40" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A41" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B41" s="1">
+        <f>-(5000*2140)/1000000</f>
+        <v>-10.7</v>
+      </c>
+      <c r="C41" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A42" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="B42" s="5">
+        <f>-SUM(B9:B11,(B13:B19),B22,B27,(B29:B34),B36:B41)</f>
+        <v>-166.32542000000001</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A43" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="B43" s="6"/>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A44" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="B44" s="5">
+        <f>ROUNDUP(SUM(B7,B42),2)</f>
+        <v>27.57</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A45" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B45" s="4">
+        <v>6</v>
+      </c>
+      <c r="C45" s="7" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A46" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B46" s="4">
+        <v>6</v>
+      </c>
+      <c r="C46" s="7" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A47" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B47" s="4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A48" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B48" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A49" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B49" s="5">
+        <f>-(B47*(B45/100) + B48*(B46/100))</f>
+        <v>-0.89999999999999991</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A50" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B50" s="5">
+        <f>B44+B49</f>
+        <v>26.67</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A51" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B51" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A52" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B52" s="5">
+        <f>MAX(0, B50-B51)</f>
+        <v>26.67</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A53" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B53" s="1">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A54" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B54" s="5">
+        <f>ROUNDUP(-B52*(B53/100),2)</f>
+        <v>-12.01</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A55" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B55" s="5">
+        <f>B50+B54</f>
+        <v>14.660000000000002</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A57" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B57" s="2"/>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A58" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B58" s="4">
+        <v>40.98</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A59" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B59" s="4">
+        <v>-3</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A60" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B60" s="5">
+        <f>B58+B59+B55</f>
+        <v>52.64</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A61" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B61" s="5">
+        <f>(B55/B58)*100</f>
+        <v>35.773548072230369</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A63" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B63" s="2"/>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A64" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B64" s="5">
+        <f>B55</f>
+        <v>14.660000000000002</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A65" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B65" s="5">
+        <f>B27</f>
+        <v>5.05</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A66" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="B66" s="5">
+        <f>B19</f>
+        <v>3.7900200000000002</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A67" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B67" s="5">
+        <f>B64+B65+B66</f>
+        <v>23.500019999999999</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A68" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B68" s="4">
+        <v>29.01</v>
+      </c>
+      <c r="C68" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A69" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B69" s="5">
+        <f>ROUNDUP(-(B7*0.2-B68),2)</f>
+        <v>-9.77</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A70" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B70" s="4">
+        <v>10.7</v>
+      </c>
+      <c r="C70" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A71" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B71" s="5">
+        <f>B67+B69+B70</f>
+        <v>24.430019999999999</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A73" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B73" s="2"/>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A74" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B74" s="6"/>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A75" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B75" s="5">
+        <f>B7*0.8</f>
+        <v>155.11427200000003</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A76" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B76" s="5">
+        <f>B68</f>
+        <v>29.01</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A77" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="B77" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A78" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="B78" s="5">
+        <f>B77+B48</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A79" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B79" s="5">
+        <f>B75+B76+B78</f>
+        <v>194.12427200000002</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A80" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B80" s="6"/>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A81" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B81" s="4">
+        <f>(70000*350)/1000000</f>
+        <v>24.5</v>
+      </c>
+      <c r="C81" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A82" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="B82" s="5">
+        <f>B10</f>
+        <v>2.64</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A83" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="B83" s="5">
+        <f>SUM(B81:B82)</f>
+        <v>27.14</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A84" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="B84" s="5">
+        <f>SUM(B13:B18,B22)</f>
+        <v>102.6104</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A85" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="B85" s="5">
+        <f>SUM(B29:B34,B36:B40,B11)</f>
+        <v>39.835000000000001</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A86" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B86" s="5">
+        <f>-B49</f>
+        <v>0.89999999999999991</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A87" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B87" s="5">
+        <f>-B54</f>
+        <v>12.01</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A88" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B88" s="4">
+        <v>21.5</v>
+      </c>
+      <c r="C88" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A89" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B89" s="4">
+        <v>4</v>
+      </c>
+      <c r="C89" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A90" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B90" s="5">
+        <f>-B59</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A91" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B91" s="5">
+        <f>SUM(B83:B90)</f>
+        <v>210.99540000000002</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A92" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B92" s="6"/>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A93" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B93" s="5">
+        <f>B79-B91</f>
+        <v>-16.871127999999999</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A94" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B94" s="4">
+        <v>26.49</v>
+      </c>
+      <c r="C94" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A95" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B95" s="5">
+        <f>B93+B94</f>
+        <v>9.6188719999999996</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="4294967293" r:id="rId1"/>
+  <ignoredErrors>
+    <ignoredError sqref="B84:B85" formulaRange="1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F22491B7-3B52-4F45-BA48-29B09780386D}">
+  <dimension ref="A1:CB95"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="57.33203125" customWidth="1"/>
+    <col min="2" max="2" width="25" customWidth="1"/>
+    <col min="3" max="3" width="153.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+    </row>
+    <row r="2" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2"/>
+    </row>
+    <row r="3" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="B3" s="10">
+        <v>55000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B4" s="4">
+        <v>3170</v>
+      </c>
+    </row>
+    <row r="5" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="B5" s="4">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="B6" s="4">
+        <v>3257.14</v>
+      </c>
+      <c r="C6" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="7" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A7" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" s="5">
+        <f>(B3*B4/1000000)+(B5*B6/1000000)</f>
+        <v>193.89284000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:80" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="C8"/>
+      <c r="D8"/>
+      <c r="E8"/>
+      <c r="F8"/>
+      <c r="G8"/>
+      <c r="H8"/>
+      <c r="I8"/>
+      <c r="J8"/>
+      <c r="K8"/>
+      <c r="L8"/>
+      <c r="M8"/>
+      <c r="N8"/>
+      <c r="O8"/>
+      <c r="P8"/>
+      <c r="Q8"/>
+      <c r="R8"/>
+      <c r="S8"/>
+      <c r="T8"/>
+      <c r="U8"/>
+      <c r="V8"/>
+      <c r="W8"/>
+      <c r="X8"/>
+      <c r="Y8"/>
+      <c r="Z8"/>
+      <c r="AA8"/>
+      <c r="AB8"/>
+      <c r="AC8"/>
+      <c r="AD8"/>
+      <c r="AE8"/>
+      <c r="AF8"/>
+      <c r="AG8"/>
+      <c r="AH8"/>
+      <c r="AI8"/>
+      <c r="AJ8"/>
+      <c r="AK8"/>
+      <c r="AL8"/>
+      <c r="AM8"/>
+      <c r="AN8"/>
+      <c r="AO8"/>
+      <c r="AP8"/>
+      <c r="AQ8"/>
+      <c r="AR8"/>
+      <c r="AS8"/>
+      <c r="AT8"/>
+      <c r="AU8"/>
+      <c r="AV8"/>
+      <c r="AW8"/>
+      <c r="AX8"/>
+      <c r="AY8"/>
+      <c r="AZ8"/>
+      <c r="BA8"/>
+      <c r="BB8"/>
+      <c r="BC8"/>
+      <c r="BD8"/>
+      <c r="BE8"/>
+      <c r="BF8"/>
+      <c r="BG8"/>
+      <c r="BH8"/>
+      <c r="BI8"/>
+      <c r="BJ8"/>
+      <c r="BK8"/>
+      <c r="BL8"/>
+      <c r="BM8"/>
+      <c r="BN8"/>
+      <c r="BO8"/>
+      <c r="BP8"/>
+      <c r="BQ8"/>
+      <c r="BR8"/>
+      <c r="BS8"/>
+      <c r="BT8"/>
+      <c r="BU8"/>
+      <c r="BV8"/>
+      <c r="BW8"/>
+      <c r="BX8"/>
+      <c r="BY8"/>
+      <c r="BZ8"/>
+      <c r="CA8"/>
+      <c r="CB8"/>
+    </row>
+    <row r="9" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A9" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B9" s="4">
+        <f>(66000*350)/1000000</f>
+        <v>23.1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="10" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A10" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B10" s="4">
+        <f>(66000*40)/1000000</f>
+        <v>2.64</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="11" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A11" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B11" s="4">
+        <f>(B3*25+B5*75)/1000000</f>
+        <v>1.825</v>
+      </c>
+      <c r="C11" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="12" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A12" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B12" s="6"/>
+      <c r="C12" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="13" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A13" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="B13" s="4">
+        <f>(((975-(975*0.05))+450)*32000)/1000000</f>
+        <v>44.04</v>
+      </c>
+      <c r="C13" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="14" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A14" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B14" s="4">
+        <f>(300*30000)/1000000</f>
+        <v>9</v>
+      </c>
+      <c r="C14" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="15" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A15" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B15" s="4">
+        <f>(((120-(120*0.05))+50)*43000)/1000000</f>
+        <v>7.0519999999999996</v>
+      </c>
+      <c r="C15" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="16" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A16" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B16" s="4">
+        <f>(((120-(120*0.05))+10)*47000)/1000000</f>
+        <v>5.8280000000000003</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="17" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A17" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="B17" s="4">
+        <f>(34*32000)/1000000</f>
+        <v>1.0880000000000001</v>
+      </c>
+    </row>
+    <row r="18" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A18" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B18" s="4">
+        <f>(510*14000+1377*1200)/1000000</f>
+        <v>8.7924000000000007</v>
+      </c>
+      <c r="C18" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="19" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A19" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="B19" s="5">
+        <f>SUM(B13:B18)*0.05</f>
+        <v>3.7900200000000002</v>
+      </c>
+      <c r="C19" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="20" spans="1:80" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="C20"/>
+      <c r="D20"/>
+      <c r="E20"/>
+      <c r="F20"/>
+      <c r="G20"/>
+      <c r="H20"/>
+      <c r="I20"/>
+      <c r="J20"/>
+      <c r="K20"/>
+      <c r="L20"/>
+      <c r="M20"/>
+      <c r="N20"/>
+      <c r="O20"/>
+      <c r="P20"/>
+      <c r="Q20"/>
+      <c r="R20"/>
+      <c r="S20"/>
+      <c r="T20"/>
+      <c r="U20"/>
+      <c r="V20"/>
+      <c r="W20"/>
+      <c r="X20"/>
+      <c r="Y20"/>
+      <c r="Z20"/>
+      <c r="AA20"/>
+      <c r="AB20"/>
+      <c r="AC20"/>
+      <c r="AD20"/>
+      <c r="AE20"/>
+      <c r="AF20"/>
+      <c r="AG20"/>
+      <c r="AH20"/>
+      <c r="AI20"/>
+      <c r="AJ20"/>
+      <c r="AK20"/>
+      <c r="AL20"/>
+      <c r="AM20"/>
+      <c r="AN20"/>
+      <c r="AO20"/>
+      <c r="AP20"/>
+      <c r="AQ20"/>
+      <c r="AR20"/>
+      <c r="AS20"/>
+      <c r="AT20"/>
+      <c r="AU20"/>
+      <c r="AV20"/>
+      <c r="AW20"/>
+      <c r="AX20"/>
+      <c r="AY20"/>
+      <c r="AZ20"/>
+      <c r="BA20"/>
+      <c r="BB20"/>
+      <c r="BC20"/>
+      <c r="BD20"/>
+      <c r="BE20"/>
+      <c r="BF20"/>
+      <c r="BG20"/>
+      <c r="BH20"/>
+      <c r="BI20"/>
+      <c r="BJ20"/>
+      <c r="BK20"/>
+      <c r="BL20"/>
+      <c r="BM20"/>
+      <c r="BN20"/>
+      <c r="BO20"/>
+      <c r="BP20"/>
+      <c r="BQ20"/>
+      <c r="BR20"/>
+      <c r="BS20"/>
+      <c r="BT20"/>
+      <c r="BU20"/>
+      <c r="BV20"/>
+      <c r="BW20"/>
+      <c r="BX20"/>
+      <c r="BY20"/>
+      <c r="BZ20"/>
+      <c r="CA20"/>
+      <c r="CB20"/>
+    </row>
+    <row r="21" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A21" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="B21" s="4">
+        <v>40</v>
+      </c>
+      <c r="C21" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="22" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A22" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="B22" s="5">
+        <f>ROUNDUP(SUM(B13:B17)*(B21/100),2)</f>
+        <v>26.810000000000002</v>
+      </c>
+    </row>
+    <row r="23" spans="1:80" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C23"/>
+      <c r="D23"/>
+      <c r="E23"/>
+      <c r="F23"/>
+      <c r="G23"/>
+      <c r="H23"/>
+      <c r="I23"/>
+      <c r="J23"/>
+      <c r="K23"/>
+      <c r="L23"/>
+      <c r="M23"/>
+      <c r="N23"/>
+      <c r="O23"/>
+      <c r="P23"/>
+      <c r="Q23"/>
+      <c r="R23"/>
+      <c r="S23"/>
+      <c r="T23"/>
+      <c r="U23"/>
+      <c r="V23"/>
+      <c r="W23"/>
+      <c r="X23"/>
+      <c r="Y23"/>
+      <c r="Z23"/>
+      <c r="AA23"/>
+      <c r="AB23"/>
+      <c r="AC23"/>
+      <c r="AD23"/>
+      <c r="AE23"/>
+      <c r="AF23"/>
+      <c r="AG23"/>
+      <c r="AH23"/>
+      <c r="AI23"/>
+      <c r="AJ23"/>
+      <c r="AK23"/>
+      <c r="AL23"/>
+      <c r="AM23"/>
+      <c r="AN23"/>
+      <c r="AO23"/>
+      <c r="AP23"/>
+      <c r="AQ23"/>
+      <c r="AR23"/>
+      <c r="AS23"/>
+      <c r="AT23"/>
+      <c r="AU23"/>
+      <c r="AV23"/>
+      <c r="AW23"/>
+      <c r="AX23"/>
+      <c r="AY23"/>
+      <c r="AZ23"/>
+      <c r="BA23"/>
+      <c r="BB23"/>
+      <c r="BC23"/>
+      <c r="BD23"/>
+      <c r="BE23"/>
+      <c r="BF23"/>
+      <c r="BG23"/>
+      <c r="BH23"/>
+      <c r="BI23"/>
+      <c r="BJ23"/>
+      <c r="BK23"/>
+      <c r="BL23"/>
+      <c r="BM23"/>
+      <c r="BN23"/>
+      <c r="BO23"/>
+      <c r="BP23"/>
+      <c r="BQ23"/>
+      <c r="BR23"/>
+      <c r="BS23"/>
+      <c r="BT23"/>
+      <c r="BU23"/>
+      <c r="BV23"/>
+      <c r="BW23"/>
+      <c r="BX23"/>
+      <c r="BY23"/>
+      <c r="BZ23"/>
+      <c r="CA23"/>
+      <c r="CB23"/>
+    </row>
+    <row r="24" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A24" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B24" s="4">
+        <v>4</v>
+      </c>
+      <c r="C24" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="25" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A25" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B25" s="4">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="26" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A26" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B26" s="1">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A27" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="B27" s="5">
+        <f>SUM(B24:B26)</f>
+        <v>5.05</v>
+      </c>
+    </row>
+    <row r="28" spans="1:80" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="B28" s="6"/>
+      <c r="C28"/>
+      <c r="D28"/>
+      <c r="E28"/>
+      <c r="F28"/>
+      <c r="G28"/>
+      <c r="H28"/>
+      <c r="I28"/>
+      <c r="J28"/>
+      <c r="K28"/>
+      <c r="L28"/>
+      <c r="M28"/>
+      <c r="N28"/>
+      <c r="O28"/>
+      <c r="P28"/>
+      <c r="Q28"/>
+      <c r="R28"/>
+      <c r="S28"/>
+      <c r="T28"/>
+      <c r="U28"/>
+      <c r="V28"/>
+      <c r="W28"/>
+      <c r="X28"/>
+      <c r="Y28"/>
+      <c r="Z28"/>
+      <c r="AA28"/>
+      <c r="AB28"/>
+      <c r="AC28"/>
+      <c r="AD28"/>
+      <c r="AE28"/>
+      <c r="AF28"/>
+      <c r="AG28"/>
+      <c r="AH28"/>
+      <c r="AI28"/>
+      <c r="AJ28"/>
+      <c r="AK28"/>
+      <c r="AL28"/>
+      <c r="AM28"/>
+      <c r="AN28"/>
+      <c r="AO28"/>
+      <c r="AP28"/>
+      <c r="AQ28"/>
+      <c r="AR28"/>
+      <c r="AS28"/>
+      <c r="AT28"/>
+      <c r="AU28"/>
+      <c r="AV28"/>
+      <c r="AW28"/>
+      <c r="AX28"/>
+      <c r="AY28"/>
+      <c r="AZ28"/>
+      <c r="BA28"/>
+      <c r="BB28"/>
+      <c r="BC28"/>
+      <c r="BD28"/>
+      <c r="BE28"/>
+      <c r="BF28"/>
+      <c r="BG28"/>
+      <c r="BH28"/>
+      <c r="BI28"/>
+      <c r="BJ28"/>
+      <c r="BK28"/>
+      <c r="BL28"/>
+      <c r="BM28"/>
+      <c r="BN28"/>
+      <c r="BO28"/>
+      <c r="BP28"/>
+      <c r="BQ28"/>
+      <c r="BR28"/>
+      <c r="BS28"/>
+      <c r="BT28"/>
+      <c r="BU28"/>
+      <c r="BV28"/>
+      <c r="BW28"/>
+      <c r="BX28"/>
+      <c r="BY28"/>
+      <c r="BZ28"/>
+      <c r="CA28"/>
+      <c r="CB28"/>
+    </row>
+    <row r="29" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A29" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="B29" s="4">
+        <v>4.75</v>
+      </c>
+      <c r="C29" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="30" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A30" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="B30" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="31" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A31" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B31" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A32" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B32" s="4">
+        <v>0.7</v>
+      </c>
+      <c r="C32" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="B33" s="4">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B34" s="4">
+        <f>(5000*100+4000*15)/1000000</f>
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="C34" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="B35" s="6"/>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B36" s="4">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="B37" s="4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A38" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B38" s="4">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="B39" s="4">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A40" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B40" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A41" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B41" s="1">
+        <f>-(5000*2140)/1000000</f>
+        <v>-10.7</v>
+      </c>
+      <c r="C41" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A42" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="B42" s="5">
+        <f>-SUM(B9:B11,(B13:B19),B22,B27,(B29:B34),B36:B41)</f>
+        <v>-166.32542000000001</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A43" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="B43" s="6"/>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A44" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="B44" s="5">
+        <f>ROUNDUP(SUM(B7,B42),2)</f>
+        <v>27.57</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A45" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B45" s="4">
+        <v>6</v>
+      </c>
+      <c r="C45" s="7" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A46" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B46" s="4">
+        <v>6</v>
+      </c>
+      <c r="C46" s="7" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A47" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B47" s="4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A48" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B48" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A49" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B49" s="5">
+        <f>-(B47*(B45/100) + B48*(B46/100))</f>
+        <v>-0.89999999999999991</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A50" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B50" s="5">
+        <f>B44+B49</f>
+        <v>26.67</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A51" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B51" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A52" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B52" s="5">
+        <f>MAX(0, B50-B51)</f>
+        <v>26.67</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A53" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B53" s="1">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A54" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B54" s="5">
+        <f>ROUNDUP(-B52*(B53/100),2)</f>
+        <v>-12.01</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A55" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B55" s="5">
+        <f>B50+B54</f>
+        <v>14.660000000000002</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A57" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B57" s="2"/>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A58" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B58" s="4">
+        <v>40.98</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A59" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B59" s="4">
+        <v>-3</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A60" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B60" s="5">
+        <f>B58+B59+B55</f>
+        <v>52.64</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A61" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B61" s="5">
+        <f>(B55/B58)*100</f>
+        <v>35.773548072230369</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A63" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B63" s="2"/>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A64" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B64" s="5">
+        <f>B55</f>
+        <v>14.660000000000002</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A65" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B65" s="5">
+        <f>B27</f>
+        <v>5.05</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A66" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="B66" s="5">
+        <f>B19</f>
+        <v>3.7900200000000002</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A67" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B67" s="5">
+        <f>B64+B65+B66</f>
+        <v>23.500019999999999</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A68" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B68" s="4">
+        <v>29.01</v>
+      </c>
+      <c r="C68" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A69" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B69" s="5">
+        <f>ROUNDUP(-(B7*0.2-B68),2)</f>
+        <v>-9.77</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A70" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B70" s="4">
+        <v>10.7</v>
+      </c>
+      <c r="C70" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A71" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B71" s="5">
+        <f>B67+B69+B70</f>
+        <v>24.430019999999999</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A73" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B73" s="2"/>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A74" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B74" s="6"/>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A75" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B75" s="5">
+        <f>B7*0.8</f>
+        <v>155.11427200000003</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A76" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B76" s="5">
+        <f>B68</f>
+        <v>29.01</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A77" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="B77" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A78" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="B78" s="5">
+        <f>B77+B48</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A79" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B79" s="5">
+        <f>B75+B76+B78</f>
+        <v>194.12427200000002</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A80" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B80" s="6"/>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A81" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B81" s="4">
+        <f>(70000*350)/1000000</f>
+        <v>24.5</v>
+      </c>
+      <c r="C81" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A82" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="B82" s="5">
+        <f>B10</f>
+        <v>2.64</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A83" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="B83" s="5">
+        <f>SUM(B81:B82)</f>
+        <v>27.14</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A84" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="B84" s="5">
+        <f>SUM(B13:B18,B22)</f>
+        <v>102.6104</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A85" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="B85" s="5">
+        <f>SUM(B29:B34,B36:B40,B11)</f>
+        <v>39.835000000000001</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A86" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B86" s="5">
+        <f>-B49</f>
+        <v>0.89999999999999991</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A87" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B87" s="5">
+        <f>-B54</f>
+        <v>12.01</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A88" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B88" s="4">
+        <v>21.5</v>
+      </c>
+      <c r="C88" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A89" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B89" s="4">
+        <v>4</v>
+      </c>
+      <c r="C89" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A90" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B90" s="5">
+        <f>-B59</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A91" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B91" s="5">
+        <f>SUM(B83:B90)</f>
+        <v>210.99540000000002</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A92" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B92" s="6"/>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A93" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B93" s="5">
+        <f>B79-B91</f>
+        <v>-16.871127999999999</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A94" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B94" s="4">
+        <v>26.49</v>
+      </c>
+      <c r="C94" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A95" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B95" s="5">
+        <f>B93+B94</f>
+        <v>9.6188719999999996</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated to planning for period 6, excel not longer in use, now: consolidated excel
</commit_message>
<xml_diff>
--- a/TOPSIM_Planungstool_V8.xlsx
+++ b/TOPSIM_Planungstool_V8.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/96db5acea2ea2686/Hochschule/Sechstes Semester/Business Simulation/Finance Tool/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="628" documentId="13_ncr:1_{F97B8132-19C7-41E8-9E6A-7064A538CFB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EA18D043-09AE-4B82-BA51-F0B4545B132D}"/>
+  <xr:revisionPtr revIDLastSave="658" documentId="13_ncr:1_{F97B8132-19C7-41E8-9E6A-7064A538CFB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{70DB080B-43A4-4B2F-8EF1-3B59EF6A0D6B}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="17496" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="17496" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sandbox Periode" sheetId="6" r:id="rId1"/>
@@ -20,6 +20,8 @@
     <sheet name="Periode 3 ALT" sheetId="4" r:id="rId5"/>
     <sheet name="Periode 3" sheetId="8" r:id="rId6"/>
     <sheet name="Periode 4" sheetId="10" r:id="rId7"/>
+    <sheet name="Periode 5 DRAFT" sheetId="11" r:id="rId8"/>
+    <sheet name="Periode 6" sheetId="12" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="629" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="869" uniqueCount="146">
   <si>
     <t>Position</t>
   </si>
@@ -6925,4 +6927,2328 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="4294967293" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E27D78C0-980F-47DC-B180-057BCC014314}">
+  <dimension ref="A1:CB95"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="57.33203125" customWidth="1"/>
+    <col min="2" max="2" width="25" customWidth="1"/>
+    <col min="3" max="3" width="153.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+    </row>
+    <row r="2" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2"/>
+    </row>
+    <row r="3" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="B3" s="10">
+        <v>55000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B4" s="4">
+        <v>3170</v>
+      </c>
+    </row>
+    <row r="5" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="B5" s="4">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="B6" s="4">
+        <v>3257.14</v>
+      </c>
+      <c r="C6" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="7" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A7" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" s="5">
+        <f>(B3*B4/1000000)+(B5*B6/1000000)</f>
+        <v>193.89284000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:80" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="C8"/>
+      <c r="D8"/>
+      <c r="E8"/>
+      <c r="F8"/>
+      <c r="G8"/>
+      <c r="H8"/>
+      <c r="I8"/>
+      <c r="J8"/>
+      <c r="K8"/>
+      <c r="L8"/>
+      <c r="M8"/>
+      <c r="N8"/>
+      <c r="O8"/>
+      <c r="P8"/>
+      <c r="Q8"/>
+      <c r="R8"/>
+      <c r="S8"/>
+      <c r="T8"/>
+      <c r="U8"/>
+      <c r="V8"/>
+      <c r="W8"/>
+      <c r="X8"/>
+      <c r="Y8"/>
+      <c r="Z8"/>
+      <c r="AA8"/>
+      <c r="AB8"/>
+      <c r="AC8"/>
+      <c r="AD8"/>
+      <c r="AE8"/>
+      <c r="AF8"/>
+      <c r="AG8"/>
+      <c r="AH8"/>
+      <c r="AI8"/>
+      <c r="AJ8"/>
+      <c r="AK8"/>
+      <c r="AL8"/>
+      <c r="AM8"/>
+      <c r="AN8"/>
+      <c r="AO8"/>
+      <c r="AP8"/>
+      <c r="AQ8"/>
+      <c r="AR8"/>
+      <c r="AS8"/>
+      <c r="AT8"/>
+      <c r="AU8"/>
+      <c r="AV8"/>
+      <c r="AW8"/>
+      <c r="AX8"/>
+      <c r="AY8"/>
+      <c r="AZ8"/>
+      <c r="BA8"/>
+      <c r="BB8"/>
+      <c r="BC8"/>
+      <c r="BD8"/>
+      <c r="BE8"/>
+      <c r="BF8"/>
+      <c r="BG8"/>
+      <c r="BH8"/>
+      <c r="BI8"/>
+      <c r="BJ8"/>
+      <c r="BK8"/>
+      <c r="BL8"/>
+      <c r="BM8"/>
+      <c r="BN8"/>
+      <c r="BO8"/>
+      <c r="BP8"/>
+      <c r="BQ8"/>
+      <c r="BR8"/>
+      <c r="BS8"/>
+      <c r="BT8"/>
+      <c r="BU8"/>
+      <c r="BV8"/>
+      <c r="BW8"/>
+      <c r="BX8"/>
+      <c r="BY8"/>
+      <c r="BZ8"/>
+      <c r="CA8"/>
+      <c r="CB8"/>
+    </row>
+    <row r="9" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A9" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B9" s="4">
+        <f>(66000*350)/1000000</f>
+        <v>23.1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="10" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A10" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B10" s="4">
+        <f>(66000*40)/1000000</f>
+        <v>2.64</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="11" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A11" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B11" s="4">
+        <f>(B3*25+B5*75)/1000000</f>
+        <v>1.825</v>
+      </c>
+      <c r="C11" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="12" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A12" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B12" s="6"/>
+      <c r="C12" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="13" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A13" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="B13" s="4">
+        <f>(((975-(975*0.05))+450)*32000)/1000000</f>
+        <v>44.04</v>
+      </c>
+      <c r="C13" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="14" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A14" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B14" s="4">
+        <f>(300*30000)/1000000</f>
+        <v>9</v>
+      </c>
+      <c r="C14" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="15" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A15" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B15" s="4">
+        <f>(((120-(120*0.05))+50)*43000)/1000000</f>
+        <v>7.0519999999999996</v>
+      </c>
+      <c r="C15" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="16" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A16" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B16" s="4">
+        <f>(((120-(120*0.05))+10)*47000)/1000000</f>
+        <v>5.8280000000000003</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="17" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A17" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="B17" s="4">
+        <f>(34*32000)/1000000</f>
+        <v>1.0880000000000001</v>
+      </c>
+    </row>
+    <row r="18" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A18" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B18" s="4">
+        <f>(510*14000+1377*1200)/1000000</f>
+        <v>8.7924000000000007</v>
+      </c>
+      <c r="C18" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="19" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A19" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="B19" s="5">
+        <f>SUM(B13:B18)*0.05</f>
+        <v>3.7900200000000002</v>
+      </c>
+      <c r="C19" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="20" spans="1:80" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="C20"/>
+      <c r="D20"/>
+      <c r="E20"/>
+      <c r="F20"/>
+      <c r="G20"/>
+      <c r="H20"/>
+      <c r="I20"/>
+      <c r="J20"/>
+      <c r="K20"/>
+      <c r="L20"/>
+      <c r="M20"/>
+      <c r="N20"/>
+      <c r="O20"/>
+      <c r="P20"/>
+      <c r="Q20"/>
+      <c r="R20"/>
+      <c r="S20"/>
+      <c r="T20"/>
+      <c r="U20"/>
+      <c r="V20"/>
+      <c r="W20"/>
+      <c r="X20"/>
+      <c r="Y20"/>
+      <c r="Z20"/>
+      <c r="AA20"/>
+      <c r="AB20"/>
+      <c r="AC20"/>
+      <c r="AD20"/>
+      <c r="AE20"/>
+      <c r="AF20"/>
+      <c r="AG20"/>
+      <c r="AH20"/>
+      <c r="AI20"/>
+      <c r="AJ20"/>
+      <c r="AK20"/>
+      <c r="AL20"/>
+      <c r="AM20"/>
+      <c r="AN20"/>
+      <c r="AO20"/>
+      <c r="AP20"/>
+      <c r="AQ20"/>
+      <c r="AR20"/>
+      <c r="AS20"/>
+      <c r="AT20"/>
+      <c r="AU20"/>
+      <c r="AV20"/>
+      <c r="AW20"/>
+      <c r="AX20"/>
+      <c r="AY20"/>
+      <c r="AZ20"/>
+      <c r="BA20"/>
+      <c r="BB20"/>
+      <c r="BC20"/>
+      <c r="BD20"/>
+      <c r="BE20"/>
+      <c r="BF20"/>
+      <c r="BG20"/>
+      <c r="BH20"/>
+      <c r="BI20"/>
+      <c r="BJ20"/>
+      <c r="BK20"/>
+      <c r="BL20"/>
+      <c r="BM20"/>
+      <c r="BN20"/>
+      <c r="BO20"/>
+      <c r="BP20"/>
+      <c r="BQ20"/>
+      <c r="BR20"/>
+      <c r="BS20"/>
+      <c r="BT20"/>
+      <c r="BU20"/>
+      <c r="BV20"/>
+      <c r="BW20"/>
+      <c r="BX20"/>
+      <c r="BY20"/>
+      <c r="BZ20"/>
+      <c r="CA20"/>
+      <c r="CB20"/>
+    </row>
+    <row r="21" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A21" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="B21" s="4">
+        <v>40</v>
+      </c>
+      <c r="C21" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="22" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A22" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="B22" s="5">
+        <f>ROUNDUP(SUM(B13:B17)*(B21/100),2)</f>
+        <v>26.810000000000002</v>
+      </c>
+    </row>
+    <row r="23" spans="1:80" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C23"/>
+      <c r="D23"/>
+      <c r="E23"/>
+      <c r="F23"/>
+      <c r="G23"/>
+      <c r="H23"/>
+      <c r="I23"/>
+      <c r="J23"/>
+      <c r="K23"/>
+      <c r="L23"/>
+      <c r="M23"/>
+      <c r="N23"/>
+      <c r="O23"/>
+      <c r="P23"/>
+      <c r="Q23"/>
+      <c r="R23"/>
+      <c r="S23"/>
+      <c r="T23"/>
+      <c r="U23"/>
+      <c r="V23"/>
+      <c r="W23"/>
+      <c r="X23"/>
+      <c r="Y23"/>
+      <c r="Z23"/>
+      <c r="AA23"/>
+      <c r="AB23"/>
+      <c r="AC23"/>
+      <c r="AD23"/>
+      <c r="AE23"/>
+      <c r="AF23"/>
+      <c r="AG23"/>
+      <c r="AH23"/>
+      <c r="AI23"/>
+      <c r="AJ23"/>
+      <c r="AK23"/>
+      <c r="AL23"/>
+      <c r="AM23"/>
+      <c r="AN23"/>
+      <c r="AO23"/>
+      <c r="AP23"/>
+      <c r="AQ23"/>
+      <c r="AR23"/>
+      <c r="AS23"/>
+      <c r="AT23"/>
+      <c r="AU23"/>
+      <c r="AV23"/>
+      <c r="AW23"/>
+      <c r="AX23"/>
+      <c r="AY23"/>
+      <c r="AZ23"/>
+      <c r="BA23"/>
+      <c r="BB23"/>
+      <c r="BC23"/>
+      <c r="BD23"/>
+      <c r="BE23"/>
+      <c r="BF23"/>
+      <c r="BG23"/>
+      <c r="BH23"/>
+      <c r="BI23"/>
+      <c r="BJ23"/>
+      <c r="BK23"/>
+      <c r="BL23"/>
+      <c r="BM23"/>
+      <c r="BN23"/>
+      <c r="BO23"/>
+      <c r="BP23"/>
+      <c r="BQ23"/>
+      <c r="BR23"/>
+      <c r="BS23"/>
+      <c r="BT23"/>
+      <c r="BU23"/>
+      <c r="BV23"/>
+      <c r="BW23"/>
+      <c r="BX23"/>
+      <c r="BY23"/>
+      <c r="BZ23"/>
+      <c r="CA23"/>
+      <c r="CB23"/>
+    </row>
+    <row r="24" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A24" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B24" s="4">
+        <v>4</v>
+      </c>
+      <c r="C24" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="25" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A25" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B25" s="4">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="26" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A26" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B26" s="1">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A27" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="B27" s="5">
+        <f>SUM(B24:B26)</f>
+        <v>5.05</v>
+      </c>
+    </row>
+    <row r="28" spans="1:80" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="B28" s="6"/>
+      <c r="C28"/>
+      <c r="D28"/>
+      <c r="E28"/>
+      <c r="F28"/>
+      <c r="G28"/>
+      <c r="H28"/>
+      <c r="I28"/>
+      <c r="J28"/>
+      <c r="K28"/>
+      <c r="L28"/>
+      <c r="M28"/>
+      <c r="N28"/>
+      <c r="O28"/>
+      <c r="P28"/>
+      <c r="Q28"/>
+      <c r="R28"/>
+      <c r="S28"/>
+      <c r="T28"/>
+      <c r="U28"/>
+      <c r="V28"/>
+      <c r="W28"/>
+      <c r="X28"/>
+      <c r="Y28"/>
+      <c r="Z28"/>
+      <c r="AA28"/>
+      <c r="AB28"/>
+      <c r="AC28"/>
+      <c r="AD28"/>
+      <c r="AE28"/>
+      <c r="AF28"/>
+      <c r="AG28"/>
+      <c r="AH28"/>
+      <c r="AI28"/>
+      <c r="AJ28"/>
+      <c r="AK28"/>
+      <c r="AL28"/>
+      <c r="AM28"/>
+      <c r="AN28"/>
+      <c r="AO28"/>
+      <c r="AP28"/>
+      <c r="AQ28"/>
+      <c r="AR28"/>
+      <c r="AS28"/>
+      <c r="AT28"/>
+      <c r="AU28"/>
+      <c r="AV28"/>
+      <c r="AW28"/>
+      <c r="AX28"/>
+      <c r="AY28"/>
+      <c r="AZ28"/>
+      <c r="BA28"/>
+      <c r="BB28"/>
+      <c r="BC28"/>
+      <c r="BD28"/>
+      <c r="BE28"/>
+      <c r="BF28"/>
+      <c r="BG28"/>
+      <c r="BH28"/>
+      <c r="BI28"/>
+      <c r="BJ28"/>
+      <c r="BK28"/>
+      <c r="BL28"/>
+      <c r="BM28"/>
+      <c r="BN28"/>
+      <c r="BO28"/>
+      <c r="BP28"/>
+      <c r="BQ28"/>
+      <c r="BR28"/>
+      <c r="BS28"/>
+      <c r="BT28"/>
+      <c r="BU28"/>
+      <c r="BV28"/>
+      <c r="BW28"/>
+      <c r="BX28"/>
+      <c r="BY28"/>
+      <c r="BZ28"/>
+      <c r="CA28"/>
+      <c r="CB28"/>
+    </row>
+    <row r="29" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A29" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="B29" s="4">
+        <v>4.75</v>
+      </c>
+      <c r="C29" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="30" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A30" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="B30" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="31" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A31" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B31" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A32" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B32" s="4">
+        <v>0.7</v>
+      </c>
+      <c r="C32" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="B33" s="4">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B34" s="4">
+        <f>(5000*100+4000*15)/1000000</f>
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="C34" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="B35" s="6"/>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B36" s="4">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="B37" s="4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A38" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B38" s="4">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="B39" s="4">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A40" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B40" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A41" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B41" s="1">
+        <f>-(5000*2140)/1000000</f>
+        <v>-10.7</v>
+      </c>
+      <c r="C41" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A42" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="B42" s="5">
+        <f>-SUM(B9:B11,(B13:B19),B22,B27,(B29:B34),B36:B41)</f>
+        <v>-166.32542000000001</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A43" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="B43" s="6"/>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A44" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="B44" s="5">
+        <f>ROUNDUP(SUM(B7,B42),2)</f>
+        <v>27.57</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A45" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B45" s="4">
+        <v>6</v>
+      </c>
+      <c r="C45" s="7" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A46" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B46" s="4">
+        <v>6</v>
+      </c>
+      <c r="C46" s="7" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A47" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B47" s="4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A48" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B48" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A49" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B49" s="5">
+        <f>-(B47*(B45/100) + B48*(B46/100))</f>
+        <v>-0.89999999999999991</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A50" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B50" s="5">
+        <f>B44+B49</f>
+        <v>26.67</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A51" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B51" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A52" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B52" s="5">
+        <f>MAX(0, B50-B51)</f>
+        <v>26.67</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A53" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B53" s="1">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A54" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B54" s="5">
+        <f>ROUNDUP(-B52*(B53/100),2)</f>
+        <v>-12.01</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A55" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B55" s="5">
+        <f>B50+B54</f>
+        <v>14.660000000000002</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A57" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B57" s="2"/>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A58" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B58" s="4">
+        <v>40.98</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A59" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B59" s="4">
+        <v>-3</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A60" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B60" s="5">
+        <f>B58+B59+B55</f>
+        <v>52.64</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A61" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B61" s="5">
+        <f>(B55/B58)*100</f>
+        <v>35.773548072230369</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A63" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B63" s="2"/>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A64" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B64" s="5">
+        <f>B55</f>
+        <v>14.660000000000002</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A65" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B65" s="5">
+        <f>B27</f>
+        <v>5.05</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A66" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="B66" s="5">
+        <f>B19</f>
+        <v>3.7900200000000002</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A67" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B67" s="5">
+        <f>B64+B65+B66</f>
+        <v>23.500019999999999</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A68" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B68" s="4">
+        <v>29.01</v>
+      </c>
+      <c r="C68" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A69" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B69" s="5">
+        <f>ROUNDUP(-(B7*0.2-B68),2)</f>
+        <v>-9.77</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A70" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B70" s="4">
+        <v>10.7</v>
+      </c>
+      <c r="C70" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A71" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B71" s="5">
+        <f>B67+B69+B70</f>
+        <v>24.430019999999999</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A73" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B73" s="2"/>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A74" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B74" s="6"/>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A75" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B75" s="5">
+        <f>B7*0.8</f>
+        <v>155.11427200000003</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A76" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B76" s="5">
+        <f>B68</f>
+        <v>29.01</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A77" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="B77" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A78" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="B78" s="5">
+        <f>B77+B48</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A79" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B79" s="5">
+        <f>B75+B76+B78</f>
+        <v>194.12427200000002</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A80" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B80" s="6"/>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A81" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B81" s="4">
+        <f>(70000*350)/1000000</f>
+        <v>24.5</v>
+      </c>
+      <c r="C81" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A82" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="B82" s="5">
+        <f>B10</f>
+        <v>2.64</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A83" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="B83" s="5">
+        <f>SUM(B81:B82)</f>
+        <v>27.14</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A84" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="B84" s="5">
+        <f>SUM(B13:B18,B22)</f>
+        <v>102.6104</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A85" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="B85" s="5">
+        <f>SUM(B29:B34,B36:B40,B11)</f>
+        <v>39.835000000000001</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A86" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B86" s="5">
+        <f>-B49</f>
+        <v>0.89999999999999991</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A87" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B87" s="5">
+        <f>-B54</f>
+        <v>12.01</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A88" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B88" s="4">
+        <v>21.5</v>
+      </c>
+      <c r="C88" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A89" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B89" s="4">
+        <v>4</v>
+      </c>
+      <c r="C89" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A90" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B90" s="5">
+        <f>-B59</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A91" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B91" s="5">
+        <f>SUM(B83:B90)</f>
+        <v>210.99540000000002</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A92" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B92" s="6"/>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A93" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B93" s="5">
+        <f>B79-B91</f>
+        <v>-16.871127999999999</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A94" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B94" s="4">
+        <v>26.49</v>
+      </c>
+      <c r="C94" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A95" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B95" s="5">
+        <f>B93+B94</f>
+        <v>9.6188719999999996</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="4294967293" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F13159E-BFC9-4123-BC4A-CE4CD46F5094}">
+  <dimension ref="A1:CB95"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="57.33203125" customWidth="1"/>
+    <col min="2" max="2" width="25" customWidth="1"/>
+    <col min="3" max="3" width="153.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+    </row>
+    <row r="2" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2"/>
+    </row>
+    <row r="3" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="B3" s="10">
+        <v>55000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B4" s="4">
+        <v>3170</v>
+      </c>
+    </row>
+    <row r="5" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="B5" s="4">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="B6" s="4">
+        <v>3257.14</v>
+      </c>
+      <c r="C6" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="7" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A7" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" s="5">
+        <f>(B3*B4/1000000)+(B5*B6/1000000)</f>
+        <v>193.89284000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:80" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="C8"/>
+      <c r="D8"/>
+      <c r="E8"/>
+      <c r="F8"/>
+      <c r="G8"/>
+      <c r="H8"/>
+      <c r="I8"/>
+      <c r="J8"/>
+      <c r="K8"/>
+      <c r="L8"/>
+      <c r="M8"/>
+      <c r="N8"/>
+      <c r="O8"/>
+      <c r="P8"/>
+      <c r="Q8"/>
+      <c r="R8"/>
+      <c r="S8"/>
+      <c r="T8"/>
+      <c r="U8"/>
+      <c r="V8"/>
+      <c r="W8"/>
+      <c r="X8"/>
+      <c r="Y8"/>
+      <c r="Z8"/>
+      <c r="AA8"/>
+      <c r="AB8"/>
+      <c r="AC8"/>
+      <c r="AD8"/>
+      <c r="AE8"/>
+      <c r="AF8"/>
+      <c r="AG8"/>
+      <c r="AH8"/>
+      <c r="AI8"/>
+      <c r="AJ8"/>
+      <c r="AK8"/>
+      <c r="AL8"/>
+      <c r="AM8"/>
+      <c r="AN8"/>
+      <c r="AO8"/>
+      <c r="AP8"/>
+      <c r="AQ8"/>
+      <c r="AR8"/>
+      <c r="AS8"/>
+      <c r="AT8"/>
+      <c r="AU8"/>
+      <c r="AV8"/>
+      <c r="AW8"/>
+      <c r="AX8"/>
+      <c r="AY8"/>
+      <c r="AZ8"/>
+      <c r="BA8"/>
+      <c r="BB8"/>
+      <c r="BC8"/>
+      <c r="BD8"/>
+      <c r="BE8"/>
+      <c r="BF8"/>
+      <c r="BG8"/>
+      <c r="BH8"/>
+      <c r="BI8"/>
+      <c r="BJ8"/>
+      <c r="BK8"/>
+      <c r="BL8"/>
+      <c r="BM8"/>
+      <c r="BN8"/>
+      <c r="BO8"/>
+      <c r="BP8"/>
+      <c r="BQ8"/>
+      <c r="BR8"/>
+      <c r="BS8"/>
+      <c r="BT8"/>
+      <c r="BU8"/>
+      <c r="BV8"/>
+      <c r="BW8"/>
+      <c r="BX8"/>
+      <c r="BY8"/>
+      <c r="BZ8"/>
+      <c r="CA8"/>
+      <c r="CB8"/>
+    </row>
+    <row r="9" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A9" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B9" s="4">
+        <f>(66000*350)/1000000</f>
+        <v>23.1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="10" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A10" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B10" s="4">
+        <f>(66000*40)/1000000</f>
+        <v>2.64</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="11" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A11" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B11" s="4">
+        <f>(B3*25+B5*75)/1000000</f>
+        <v>1.825</v>
+      </c>
+      <c r="C11" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="12" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A12" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B12" s="6"/>
+      <c r="C12" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="13" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A13" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="B13" s="4">
+        <f>(((975-(975*0.05))+450)*32000)/1000000</f>
+        <v>44.04</v>
+      </c>
+      <c r="C13" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="14" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A14" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B14" s="4">
+        <f>(300*30000)/1000000</f>
+        <v>9</v>
+      </c>
+      <c r="C14" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="15" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A15" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B15" s="4">
+        <f>(((120-(120*0.05))+50)*43000)/1000000</f>
+        <v>7.0519999999999996</v>
+      </c>
+      <c r="C15" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="16" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A16" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B16" s="4">
+        <f>(((120-(120*0.05))+10)*47000)/1000000</f>
+        <v>5.8280000000000003</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="17" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A17" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="B17" s="4">
+        <f>(34*32000)/1000000</f>
+        <v>1.0880000000000001</v>
+      </c>
+    </row>
+    <row r="18" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A18" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B18" s="4">
+        <f>(510*14000+1377*1200)/1000000</f>
+        <v>8.7924000000000007</v>
+      </c>
+      <c r="C18" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="19" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A19" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="B19" s="5">
+        <f>SUM(B13:B18)*0.05</f>
+        <v>3.7900200000000002</v>
+      </c>
+      <c r="C19" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="20" spans="1:80" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="C20"/>
+      <c r="D20"/>
+      <c r="E20"/>
+      <c r="F20"/>
+      <c r="G20"/>
+      <c r="H20"/>
+      <c r="I20"/>
+      <c r="J20"/>
+      <c r="K20"/>
+      <c r="L20"/>
+      <c r="M20"/>
+      <c r="N20"/>
+      <c r="O20"/>
+      <c r="P20"/>
+      <c r="Q20"/>
+      <c r="R20"/>
+      <c r="S20"/>
+      <c r="T20"/>
+      <c r="U20"/>
+      <c r="V20"/>
+      <c r="W20"/>
+      <c r="X20"/>
+      <c r="Y20"/>
+      <c r="Z20"/>
+      <c r="AA20"/>
+      <c r="AB20"/>
+      <c r="AC20"/>
+      <c r="AD20"/>
+      <c r="AE20"/>
+      <c r="AF20"/>
+      <c r="AG20"/>
+      <c r="AH20"/>
+      <c r="AI20"/>
+      <c r="AJ20"/>
+      <c r="AK20"/>
+      <c r="AL20"/>
+      <c r="AM20"/>
+      <c r="AN20"/>
+      <c r="AO20"/>
+      <c r="AP20"/>
+      <c r="AQ20"/>
+      <c r="AR20"/>
+      <c r="AS20"/>
+      <c r="AT20"/>
+      <c r="AU20"/>
+      <c r="AV20"/>
+      <c r="AW20"/>
+      <c r="AX20"/>
+      <c r="AY20"/>
+      <c r="AZ20"/>
+      <c r="BA20"/>
+      <c r="BB20"/>
+      <c r="BC20"/>
+      <c r="BD20"/>
+      <c r="BE20"/>
+      <c r="BF20"/>
+      <c r="BG20"/>
+      <c r="BH20"/>
+      <c r="BI20"/>
+      <c r="BJ20"/>
+      <c r="BK20"/>
+      <c r="BL20"/>
+      <c r="BM20"/>
+      <c r="BN20"/>
+      <c r="BO20"/>
+      <c r="BP20"/>
+      <c r="BQ20"/>
+      <c r="BR20"/>
+      <c r="BS20"/>
+      <c r="BT20"/>
+      <c r="BU20"/>
+      <c r="BV20"/>
+      <c r="BW20"/>
+      <c r="BX20"/>
+      <c r="BY20"/>
+      <c r="BZ20"/>
+      <c r="CA20"/>
+      <c r="CB20"/>
+    </row>
+    <row r="21" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A21" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="B21" s="4">
+        <v>40</v>
+      </c>
+      <c r="C21" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="22" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A22" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="B22" s="5">
+        <f>ROUNDUP(SUM(B13:B17)*(B21/100),2)</f>
+        <v>26.810000000000002</v>
+      </c>
+    </row>
+    <row r="23" spans="1:80" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C23"/>
+      <c r="D23"/>
+      <c r="E23"/>
+      <c r="F23"/>
+      <c r="G23"/>
+      <c r="H23"/>
+      <c r="I23"/>
+      <c r="J23"/>
+      <c r="K23"/>
+      <c r="L23"/>
+      <c r="M23"/>
+      <c r="N23"/>
+      <c r="O23"/>
+      <c r="P23"/>
+      <c r="Q23"/>
+      <c r="R23"/>
+      <c r="S23"/>
+      <c r="T23"/>
+      <c r="U23"/>
+      <c r="V23"/>
+      <c r="W23"/>
+      <c r="X23"/>
+      <c r="Y23"/>
+      <c r="Z23"/>
+      <c r="AA23"/>
+      <c r="AB23"/>
+      <c r="AC23"/>
+      <c r="AD23"/>
+      <c r="AE23"/>
+      <c r="AF23"/>
+      <c r="AG23"/>
+      <c r="AH23"/>
+      <c r="AI23"/>
+      <c r="AJ23"/>
+      <c r="AK23"/>
+      <c r="AL23"/>
+      <c r="AM23"/>
+      <c r="AN23"/>
+      <c r="AO23"/>
+      <c r="AP23"/>
+      <c r="AQ23"/>
+      <c r="AR23"/>
+      <c r="AS23"/>
+      <c r="AT23"/>
+      <c r="AU23"/>
+      <c r="AV23"/>
+      <c r="AW23"/>
+      <c r="AX23"/>
+      <c r="AY23"/>
+      <c r="AZ23"/>
+      <c r="BA23"/>
+      <c r="BB23"/>
+      <c r="BC23"/>
+      <c r="BD23"/>
+      <c r="BE23"/>
+      <c r="BF23"/>
+      <c r="BG23"/>
+      <c r="BH23"/>
+      <c r="BI23"/>
+      <c r="BJ23"/>
+      <c r="BK23"/>
+      <c r="BL23"/>
+      <c r="BM23"/>
+      <c r="BN23"/>
+      <c r="BO23"/>
+      <c r="BP23"/>
+      <c r="BQ23"/>
+      <c r="BR23"/>
+      <c r="BS23"/>
+      <c r="BT23"/>
+      <c r="BU23"/>
+      <c r="BV23"/>
+      <c r="BW23"/>
+      <c r="BX23"/>
+      <c r="BY23"/>
+      <c r="BZ23"/>
+      <c r="CA23"/>
+      <c r="CB23"/>
+    </row>
+    <row r="24" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A24" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B24" s="4">
+        <v>4</v>
+      </c>
+      <c r="C24" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="25" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A25" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B25" s="4">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="26" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A26" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B26" s="1">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A27" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="B27" s="5">
+        <f>SUM(B24:B26)</f>
+        <v>5.05</v>
+      </c>
+    </row>
+    <row r="28" spans="1:80" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="B28" s="6"/>
+      <c r="C28"/>
+      <c r="D28"/>
+      <c r="E28"/>
+      <c r="F28"/>
+      <c r="G28"/>
+      <c r="H28"/>
+      <c r="I28"/>
+      <c r="J28"/>
+      <c r="K28"/>
+      <c r="L28"/>
+      <c r="M28"/>
+      <c r="N28"/>
+      <c r="O28"/>
+      <c r="P28"/>
+      <c r="Q28"/>
+      <c r="R28"/>
+      <c r="S28"/>
+      <c r="T28"/>
+      <c r="U28"/>
+      <c r="V28"/>
+      <c r="W28"/>
+      <c r="X28"/>
+      <c r="Y28"/>
+      <c r="Z28"/>
+      <c r="AA28"/>
+      <c r="AB28"/>
+      <c r="AC28"/>
+      <c r="AD28"/>
+      <c r="AE28"/>
+      <c r="AF28"/>
+      <c r="AG28"/>
+      <c r="AH28"/>
+      <c r="AI28"/>
+      <c r="AJ28"/>
+      <c r="AK28"/>
+      <c r="AL28"/>
+      <c r="AM28"/>
+      <c r="AN28"/>
+      <c r="AO28"/>
+      <c r="AP28"/>
+      <c r="AQ28"/>
+      <c r="AR28"/>
+      <c r="AS28"/>
+      <c r="AT28"/>
+      <c r="AU28"/>
+      <c r="AV28"/>
+      <c r="AW28"/>
+      <c r="AX28"/>
+      <c r="AY28"/>
+      <c r="AZ28"/>
+      <c r="BA28"/>
+      <c r="BB28"/>
+      <c r="BC28"/>
+      <c r="BD28"/>
+      <c r="BE28"/>
+      <c r="BF28"/>
+      <c r="BG28"/>
+      <c r="BH28"/>
+      <c r="BI28"/>
+      <c r="BJ28"/>
+      <c r="BK28"/>
+      <c r="BL28"/>
+      <c r="BM28"/>
+      <c r="BN28"/>
+      <c r="BO28"/>
+      <c r="BP28"/>
+      <c r="BQ28"/>
+      <c r="BR28"/>
+      <c r="BS28"/>
+      <c r="BT28"/>
+      <c r="BU28"/>
+      <c r="BV28"/>
+      <c r="BW28"/>
+      <c r="BX28"/>
+      <c r="BY28"/>
+      <c r="BZ28"/>
+      <c r="CA28"/>
+      <c r="CB28"/>
+    </row>
+    <row r="29" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A29" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="B29" s="4">
+        <v>4.75</v>
+      </c>
+      <c r="C29" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="30" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A30" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="B30" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="31" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A31" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B31" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:80" x14ac:dyDescent="0.3">
+      <c r="A32" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B32" s="4">
+        <v>0.7</v>
+      </c>
+      <c r="C32" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="B33" s="4">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B34" s="4">
+        <f>(5000*100+4000*15)/1000000</f>
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="C34" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="B35" s="6"/>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B36" s="4">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="B37" s="4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A38" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B38" s="4">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="B39" s="4">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A40" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B40" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A41" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B41" s="1">
+        <f>-(5000*2140)/1000000</f>
+        <v>-10.7</v>
+      </c>
+      <c r="C41" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A42" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="B42" s="5">
+        <f>-SUM(B9:B11,(B13:B19),B22,B27,(B29:B34),B36:B41)</f>
+        <v>-166.32542000000001</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A43" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="B43" s="6"/>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A44" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="B44" s="5">
+        <f>ROUNDUP(SUM(B7,B42),2)</f>
+        <v>27.57</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A45" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B45" s="4">
+        <v>6</v>
+      </c>
+      <c r="C45" s="7" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A46" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B46" s="4">
+        <v>6</v>
+      </c>
+      <c r="C46" s="7" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A47" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B47" s="4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A48" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B48" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A49" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B49" s="5">
+        <f>-(B47*(B45/100) + B48*(B46/100))</f>
+        <v>-0.89999999999999991</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A50" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B50" s="5">
+        <f>B44+B49</f>
+        <v>26.67</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A51" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B51" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A52" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B52" s="5">
+        <f>MAX(0, B50-B51)</f>
+        <v>26.67</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A53" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B53" s="1">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A54" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B54" s="5">
+        <f>ROUNDUP(-B52*(B53/100),2)</f>
+        <v>-12.01</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A55" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B55" s="5">
+        <f>B50+B54</f>
+        <v>14.660000000000002</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A57" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B57" s="2"/>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A58" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B58" s="4">
+        <v>40.98</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A59" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B59" s="4">
+        <v>-3</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A60" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B60" s="5">
+        <f>B58+B59+B55</f>
+        <v>52.64</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A61" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B61" s="5">
+        <f>(B55/B58)*100</f>
+        <v>35.773548072230369</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A63" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B63" s="2"/>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A64" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B64" s="5">
+        <f>B55</f>
+        <v>14.660000000000002</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A65" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B65" s="5">
+        <f>B27</f>
+        <v>5.05</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A66" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="B66" s="5">
+        <f>B19</f>
+        <v>3.7900200000000002</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A67" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B67" s="5">
+        <f>B64+B65+B66</f>
+        <v>23.500019999999999</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A68" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B68" s="4">
+        <v>29.01</v>
+      </c>
+      <c r="C68" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A69" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B69" s="5">
+        <f>ROUNDUP(-(B7*0.2-B68),2)</f>
+        <v>-9.77</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A70" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B70" s="4">
+        <v>10.7</v>
+      </c>
+      <c r="C70" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A71" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B71" s="5">
+        <f>B67+B69+B70</f>
+        <v>24.430019999999999</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A73" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B73" s="2"/>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A74" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B74" s="6"/>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A75" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B75" s="5">
+        <f>B7*0.8</f>
+        <v>155.11427200000003</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A76" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B76" s="5">
+        <f>B68</f>
+        <v>29.01</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A77" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="B77" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A78" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="B78" s="5">
+        <f>B77+B48</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A79" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B79" s="5">
+        <f>B75+B76+B78</f>
+        <v>194.12427200000002</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A80" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B80" s="6"/>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A81" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B81" s="4">
+        <f>(70000*350)/1000000</f>
+        <v>24.5</v>
+      </c>
+      <c r="C81" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A82" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="B82" s="5">
+        <f>B10</f>
+        <v>2.64</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A83" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="B83" s="5">
+        <f>SUM(B81:B82)</f>
+        <v>27.14</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A84" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="B84" s="5">
+        <f>SUM(B13:B18,B22)</f>
+        <v>102.6104</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A85" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="B85" s="5">
+        <f>SUM(B29:B34,B36:B40,B11)</f>
+        <v>39.835000000000001</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A86" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B86" s="5">
+        <f>-B49</f>
+        <v>0.89999999999999991</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A87" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B87" s="5">
+        <f>-B54</f>
+        <v>12.01</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A88" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B88" s="4">
+        <v>21.5</v>
+      </c>
+      <c r="C88" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A89" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B89" s="4">
+        <v>4</v>
+      </c>
+      <c r="C89" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A90" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B90" s="5">
+        <f>-B59</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A91" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B91" s="5">
+        <f>SUM(B83:B90)</f>
+        <v>210.99540000000002</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A92" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B92" s="6"/>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A93" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B93" s="5">
+        <f>B79-B91</f>
+        <v>-16.871127999999999</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A94" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B94" s="4">
+        <v>26.49</v>
+      </c>
+      <c r="C94" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A95" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B95" s="5">
+        <f>B93+B94</f>
+        <v>9.6188719999999996</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="4294967293" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>